<commit_message>
Improve training and prediction job polling
</commit_message>
<xml_diff>
--- a/预测文件/预测文件.xlsx
+++ b/预测文件/预测文件.xlsx
@@ -1107,10 +1107,8 @@
           <t>37445</t>
         </is>
       </c>
-      <c r="J2" s="0" t="inlineStr">
-        <is>
-          <t>285.8835</t>
-        </is>
+      <c r="J2" s="0" t="n">
+        <v>285.8835</v>
       </c>
     </row>
     <row r="3">
@@ -1154,10 +1152,8 @@
           <t>22596.14</t>
         </is>
       </c>
-      <c r="J3" s="0" t="inlineStr">
-        <is>
-          <t>281.5751</t>
-        </is>
+      <c r="J3" s="0" t="n">
+        <v>281.5751</v>
       </c>
     </row>
     <row r="4">
@@ -1201,10 +1197,8 @@
           <t>21935.81</t>
         </is>
       </c>
-      <c r="J4" s="0" t="inlineStr">
-        <is>
-          <t>270.7642</t>
-        </is>
+      <c r="J4" s="0" t="n">
+        <v>270.7642</v>
       </c>
     </row>
     <row r="5">
@@ -1248,10 +1242,8 @@
           <t>21354.84</t>
         </is>
       </c>
-      <c r="J5" s="0" t="inlineStr">
-        <is>
-          <t>265.2364</t>
-        </is>
+      <c r="J5" s="0" t="n">
+        <v>265.2364</v>
       </c>
     </row>
     <row r="6">
@@ -1295,10 +1287,8 @@
           <t>20709.8</t>
         </is>
       </c>
-      <c r="J6" s="0" t="inlineStr">
-        <is>
-          <t>269.3633</t>
-        </is>
+      <c r="J6" s="0" t="n">
+        <v>269.3633</v>
       </c>
     </row>
     <row r="7">
@@ -1342,10 +1332,8 @@
           <t>20188.43</t>
         </is>
       </c>
-      <c r="J7" s="0" t="inlineStr">
-        <is>
-          <t>264.7001</t>
-        </is>
+      <c r="J7" s="0" t="n">
+        <v>264.7001</v>
       </c>
     </row>
     <row r="8">
@@ -1389,10 +1377,8 @@
           <t>19752.33</t>
         </is>
       </c>
-      <c r="J8" s="0" t="inlineStr">
-        <is>
-          <t>259.7508</t>
-        </is>
+      <c r="J8" s="0" t="n">
+        <v>259.7508</v>
       </c>
     </row>
     <row r="9">
@@ -1436,10 +1422,8 @@
           <t>19181.02</t>
         </is>
       </c>
-      <c r="J9" s="0" t="inlineStr">
-        <is>
-          <t>250.9712</t>
-        </is>
+      <c r="J9" s="0" t="n">
+        <v>250.9712</v>
       </c>
     </row>
     <row r="10">
@@ -1483,10 +1467,8 @@
           <t>18798.65</t>
         </is>
       </c>
-      <c r="J10" s="0" t="inlineStr">
-        <is>
-          <t>254.1673</t>
-        </is>
+      <c r="J10" s="0" t="n">
+        <v>254.1673</v>
       </c>
     </row>
     <row r="11">
@@ -1530,10 +1512,8 @@
           <t>18461.98</t>
         </is>
       </c>
-      <c r="J11" s="0" t="inlineStr">
-        <is>
-          <t>248.5995</t>
-        </is>
+      <c r="J11" s="0" t="n">
+        <v>248.5995</v>
       </c>
     </row>
     <row r="12">
@@ -1577,10 +1557,8 @@
           <t>18248.84</t>
         </is>
       </c>
-      <c r="J12" s="0" t="inlineStr">
-        <is>
-          <t>246.4259</t>
-        </is>
+      <c r="J12" s="0" t="n">
+        <v>246.4259</v>
       </c>
     </row>
     <row r="13">
@@ -1624,10 +1602,8 @@
           <t>18106.24</t>
         </is>
       </c>
-      <c r="J13" s="0" t="inlineStr">
-        <is>
-          <t>244.5</t>
-        </is>
+      <c r="J13" s="0" t="n">
+        <v>244.5</v>
       </c>
     </row>
     <row r="14">
@@ -1671,10 +1647,8 @@
           <t>18026.29</t>
         </is>
       </c>
-      <c r="J14" s="0" t="inlineStr">
-        <is>
-          <t>242.9654</t>
-        </is>
+      <c r="J14" s="0" t="n">
+        <v>242.9654</v>
       </c>
     </row>
     <row r="15">
@@ -1718,10 +1692,8 @@
           <t>17856.79</t>
         </is>
       </c>
-      <c r="J15" s="0" t="inlineStr">
-        <is>
-          <t>241.3686</t>
-        </is>
+      <c r="J15" s="0" t="n">
+        <v>241.3686</v>
       </c>
     </row>
     <row r="16">
@@ -1765,10 +1737,8 @@
           <t>17639.33</t>
         </is>
       </c>
-      <c r="J16" s="0" t="inlineStr">
-        <is>
-          <t>237.4807</t>
-        </is>
+      <c r="J16" s="0" t="n">
+        <v>237.4807</v>
       </c>
     </row>
     <row r="17">
@@ -1812,10 +1782,8 @@
           <t>17524.57</t>
         </is>
       </c>
-      <c r="J17" s="0" t="inlineStr">
-        <is>
-          <t>239.2931</t>
-        </is>
+      <c r="J17" s="0" t="n">
+        <v>239.2931</v>
       </c>
     </row>
     <row r="18">
@@ -1859,10 +1827,8 @@
           <t>17516.25</t>
         </is>
       </c>
-      <c r="J18" s="0" t="inlineStr">
-        <is>
-          <t>239.3494</t>
-        </is>
+      <c r="J18" s="0" t="n">
+        <v>239.3494</v>
       </c>
     </row>
     <row r="19">
@@ -1906,10 +1872,8 @@
           <t>17517.67</t>
         </is>
       </c>
-      <c r="J19" s="0" t="inlineStr">
-        <is>
-          <t>239.3401</t>
-        </is>
+      <c r="J19" s="0" t="n">
+        <v>239.3401</v>
       </c>
     </row>
     <row r="20">
@@ -1953,10 +1917,8 @@
           <t>17721.03</t>
         </is>
       </c>
-      <c r="J20" s="0" t="inlineStr">
-        <is>
-          <t>241.4099</t>
-        </is>
+      <c r="J20" s="0" t="n">
+        <v>241.4099</v>
       </c>
     </row>
     <row r="21">
@@ -2000,10 +1962,8 @@
           <t>17899.22</t>
         </is>
       </c>
-      <c r="J21" s="0" t="inlineStr">
-        <is>
-          <t>241.5593</t>
-        </is>
+      <c r="J21" s="0" t="n">
+        <v>241.5593</v>
       </c>
     </row>
     <row r="22">
@@ -2047,10 +2007,8 @@
           <t>18089.5</t>
         </is>
       </c>
-      <c r="J22" s="0" t="inlineStr">
-        <is>
-          <t>245.4388</t>
-        </is>
+      <c r="J22" s="0" t="n">
+        <v>245.4388</v>
       </c>
     </row>
     <row r="23">
@@ -2094,10 +2052,8 @@
           <t>18792.66</t>
         </is>
       </c>
-      <c r="J23" s="0" t="inlineStr">
-        <is>
-          <t>256.7535</t>
-        </is>
+      <c r="J23" s="0" t="n">
+        <v>256.7535</v>
       </c>
     </row>
     <row r="24">
@@ -2141,10 +2097,8 @@
           <t>19244.24</t>
         </is>
       </c>
-      <c r="J24" s="0" t="inlineStr">
-        <is>
-          <t>253.641</t>
-        </is>
+      <c r="J24" s="0" t="n">
+        <v>253.641</v>
       </c>
     </row>
     <row r="25">
@@ -2188,10 +2142,8 @@
           <t>19940.13</t>
         </is>
       </c>
-      <c r="J25" s="0" t="inlineStr">
-        <is>
-          <t>264.5663</t>
-        </is>
+      <c r="J25" s="0" t="n">
+        <v>264.5663</v>
       </c>
     </row>
     <row r="26">
@@ -2235,10 +2187,8 @@
           <t>19989.25</t>
         </is>
       </c>
-      <c r="J26" s="0" t="inlineStr">
-        <is>
-          <t>261.3196</t>
-        </is>
+      <c r="J26" s="0" t="n">
+        <v>261.3196</v>
       </c>
     </row>
     <row r="27">
@@ -2282,10 +2232,8 @@
           <t>19389.56</t>
         </is>
       </c>
-      <c r="J27" s="0" t="inlineStr">
-        <is>
-          <t>251.6086</t>
-        </is>
+      <c r="J27" s="0" t="n">
+        <v>251.6086</v>
       </c>
     </row>
     <row r="28">
@@ -2329,10 +2277,8 @@
           <t>18097.15</t>
         </is>
       </c>
-      <c r="J28" s="0" t="inlineStr">
-        <is>
-          <t>238.1576</t>
-        </is>
+      <c r="J28" s="0" t="n">
+        <v>238.1576</v>
       </c>
     </row>
     <row r="29">
@@ -2376,10 +2322,8 @@
           <t>17060.36</t>
         </is>
       </c>
-      <c r="J29" s="0" t="inlineStr">
-        <is>
-          <t>174.6008</t>
-        </is>
+      <c r="J29" s="0" t="n">
+        <v>174.6008</v>
       </c>
     </row>
     <row r="30">
@@ -2423,10 +2367,8 @@
           <t>15930</t>
         </is>
       </c>
-      <c r="J30" s="0" t="inlineStr">
-        <is>
-          <t>152.2188</t>
-        </is>
+      <c r="J30" s="0" t="n">
+        <v>152.2188</v>
       </c>
     </row>
     <row r="31">
@@ -2470,10 +2412,8 @@
           <t>14458.28</t>
         </is>
       </c>
-      <c r="J31" s="0" t="inlineStr">
-        <is>
-          <t>134.0804</t>
-        </is>
+      <c r="J31" s="0" t="n">
+        <v>134.0804</v>
       </c>
     </row>
     <row r="32">
@@ -2517,10 +2457,8 @@
           <t>13270.07</t>
         </is>
       </c>
-      <c r="J32" s="0" t="inlineStr">
-        <is>
-          <t>43.109</t>
-        </is>
+      <c r="J32" s="0" t="n">
+        <v>43.109</v>
       </c>
     </row>
     <row r="33">
@@ -2564,10 +2502,8 @@
           <t>11922.69</t>
         </is>
       </c>
-      <c r="J33" s="0" t="inlineStr">
-        <is>
-          <t>56.939</t>
-        </is>
+      <c r="J33" s="0" t="n">
+        <v>56.939</v>
       </c>
     </row>
     <row r="34">
@@ -2611,10 +2547,8 @@
           <t>10611.72</t>
         </is>
       </c>
-      <c r="J34" s="0" t="inlineStr">
-        <is>
-          <t>26.8584</t>
-        </is>
+      <c r="J34" s="0" t="n">
+        <v>26.8584</v>
       </c>
     </row>
     <row r="35">
@@ -2658,10 +2592,8 @@
           <t>8830.05</t>
         </is>
       </c>
-      <c r="J35" s="0" t="inlineStr">
-        <is>
-          <t>35.3151</t>
-        </is>
+      <c r="J35" s="0" t="n">
+        <v>35.3151</v>
       </c>
     </row>
     <row r="36">
@@ -2705,10 +2637,8 @@
           <t>7324.51</t>
         </is>
       </c>
-      <c r="J36" s="0" t="inlineStr">
-        <is>
-          <t>2.3303</t>
-        </is>
+      <c r="J36" s="0" t="n">
+        <v>2.3303</v>
       </c>
     </row>
     <row r="37">
@@ -2752,10 +2682,8 @@
           <t>5984.99</t>
         </is>
       </c>
-      <c r="J37" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J37" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -2799,10 +2727,8 @@
           <t>4730.77</t>
         </is>
       </c>
-      <c r="J38" s="0" t="inlineStr">
-        <is>
-          <t>4.5215</t>
-        </is>
+      <c r="J38" s="0" t="n">
+        <v>4.5215</v>
       </c>
     </row>
     <row r="39">
@@ -2846,10 +2772,8 @@
           <t>3427.66</t>
         </is>
       </c>
-      <c r="J39" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J39" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -2893,10 +2817,8 @@
           <t>2181.93</t>
         </is>
       </c>
-      <c r="J40" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J40" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -2940,10 +2862,8 @@
           <t>955.619999999999</t>
         </is>
       </c>
-      <c r="J41" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J41" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -2987,10 +2907,8 @@
           <t>-167.950000000001</t>
         </is>
       </c>
-      <c r="J42" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J42" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -3034,10 +2952,8 @@
           <t>-1227.8</t>
         </is>
       </c>
-      <c r="J43" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J43" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -3081,10 +2997,8 @@
           <t>-2004.82</t>
         </is>
       </c>
-      <c r="J44" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J44" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -3128,10 +3042,8 @@
           <t>-2524.96</t>
         </is>
       </c>
-      <c r="J45" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J45" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -3175,10 +3087,8 @@
           <t>-3068.43</t>
         </is>
       </c>
-      <c r="J46" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J46" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -3222,10 +3132,8 @@
           <t>-3487.62</t>
         </is>
       </c>
-      <c r="J47" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J47" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -3269,10 +3177,8 @@
           <t>-4079.62</t>
         </is>
       </c>
-      <c r="J48" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J48" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -3316,10 +3222,8 @@
           <t>-4631.93</t>
         </is>
       </c>
-      <c r="J49" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J49" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -3363,10 +3267,8 @@
           <t>-5057.49</t>
         </is>
       </c>
-      <c r="J50" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J50" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -3410,10 +3312,8 @@
           <t>-5040.12</t>
         </is>
       </c>
-      <c r="J51" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J51" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -3457,10 +3357,8 @@
           <t>-4828.22</t>
         </is>
       </c>
-      <c r="J52" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J52" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -3504,10 +3402,8 @@
           <t>-4455.56</t>
         </is>
       </c>
-      <c r="J53" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J53" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -3551,10 +3447,8 @@
           <t>-4028.62</t>
         </is>
       </c>
-      <c r="J54" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J54" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -3598,10 +3492,8 @@
           <t>-3729.09</t>
         </is>
       </c>
-      <c r="J55" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J55" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -3645,10 +3537,8 @@
           <t>-3243.61</t>
         </is>
       </c>
-      <c r="J56" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J56" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -3692,10 +3582,8 @@
           <t>-2450.03</t>
         </is>
       </c>
-      <c r="J57" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J57" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -3739,10 +3627,8 @@
           <t>-1547.67</t>
         </is>
       </c>
-      <c r="J58" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J58" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -3786,10 +3672,8 @@
           <t>-352.77</t>
         </is>
       </c>
-      <c r="J59" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J59" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -3833,10 +3717,8 @@
           <t>836.649999999998</t>
         </is>
       </c>
-      <c r="J60" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J60" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -3880,10 +3762,8 @@
           <t>1760.94</t>
         </is>
       </c>
-      <c r="J61" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J61" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -3927,10 +3807,8 @@
           <t>3177.5</t>
         </is>
       </c>
-      <c r="J62" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J62" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -3974,10 +3852,8 @@
           <t>4645.41</t>
         </is>
       </c>
-      <c r="J63" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J63" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -4021,10 +3897,8 @@
           <t>6152.55</t>
         </is>
       </c>
-      <c r="J64" s="0" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="J64" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -4068,10 +3942,8 @@
           <t>7555.98</t>
         </is>
       </c>
-      <c r="J65" s="0" t="inlineStr">
-        <is>
-          <t>5.5346</t>
-        </is>
+      <c r="J65" s="0" t="n">
+        <v>5.5346</v>
       </c>
     </row>
     <row r="66">
@@ -4115,10 +3987,8 @@
           <t>9058.79</t>
         </is>
       </c>
-      <c r="J66" s="0" t="inlineStr">
-        <is>
-          <t>8.3987</t>
-        </is>
+      <c r="J66" s="0" t="n">
+        <v>8.3987</v>
       </c>
     </row>
     <row r="67">
@@ -4162,10 +4032,8 @@
           <t>10629.75</t>
         </is>
       </c>
-      <c r="J67" s="0" t="inlineStr">
-        <is>
-          <t>9.6511</t>
-        </is>
+      <c r="J67" s="0" t="n">
+        <v>9.6511</v>
       </c>
     </row>
     <row r="68">
@@ -4209,10 +4077,8 @@
           <t>12650.77</t>
         </is>
       </c>
-      <c r="J68" s="0" t="inlineStr">
-        <is>
-          <t>55.6459</t>
-        </is>
+      <c r="J68" s="0" t="n">
+        <v>55.6459</v>
       </c>
     </row>
     <row r="69">
@@ -4256,10 +4122,8 @@
           <t>14735.77</t>
         </is>
       </c>
-      <c r="J69" s="0" t="inlineStr">
-        <is>
-          <t>110.2572</t>
-        </is>
+      <c r="J69" s="0" t="n">
+        <v>110.2572</v>
       </c>
     </row>
     <row r="70">
@@ -4303,10 +4167,8 @@
           <t>16562.72</t>
         </is>
       </c>
-      <c r="J70" s="0" t="inlineStr">
-        <is>
-          <t>63.1874</t>
-        </is>
+      <c r="J70" s="0" t="n">
+        <v>63.1874</v>
       </c>
     </row>
     <row r="71">
@@ -4350,10 +4212,8 @@
           <t>18583.24</t>
         </is>
       </c>
-      <c r="J71" s="0" t="inlineStr">
-        <is>
-          <t>231.1111</t>
-        </is>
+      <c r="J71" s="0" t="n">
+        <v>231.1111</v>
       </c>
     </row>
     <row r="72">
@@ -4397,10 +4257,8 @@
           <t>20489.77</t>
         </is>
       </c>
-      <c r="J72" s="0" t="inlineStr">
-        <is>
-          <t>247.4391</t>
-        </is>
+      <c r="J72" s="0" t="n">
+        <v>247.4391</v>
       </c>
     </row>
     <row r="73">
@@ -4444,10 +4302,8 @@
           <t>22465.65</t>
         </is>
       </c>
-      <c r="J73" s="0" t="inlineStr">
-        <is>
-          <t>264.0113</t>
-        </is>
+      <c r="J73" s="0" t="n">
+        <v>264.0113</v>
       </c>
     </row>
     <row r="74">
@@ -4491,10 +4347,8 @@
           <t>24428.79</t>
         </is>
       </c>
-      <c r="J74" s="0" t="inlineStr">
-        <is>
-          <t>269.9186</t>
-        </is>
+      <c r="J74" s="0" t="n">
+        <v>269.9186</v>
       </c>
     </row>
     <row r="75">
@@ -4538,10 +4392,8 @@
           <t>26058.83</t>
         </is>
       </c>
-      <c r="J75" s="0" t="inlineStr">
-        <is>
-          <t>293.4086</t>
-        </is>
+      <c r="J75" s="0" t="n">
+        <v>293.4086</v>
       </c>
     </row>
     <row r="76">
@@ -4585,10 +4437,8 @@
           <t>27430.47</t>
         </is>
       </c>
-      <c r="J76" s="0" t="inlineStr">
-        <is>
-          <t>333.4358</t>
-        </is>
+      <c r="J76" s="0" t="n">
+        <v>333.4358</v>
       </c>
     </row>
     <row r="77">
@@ -4632,10 +4482,8 @@
           <t>28606.62</t>
         </is>
       </c>
-      <c r="J77" s="0" t="inlineStr">
-        <is>
-          <t>364.6738</t>
-        </is>
+      <c r="J77" s="0" t="n">
+        <v>364.6738</v>
       </c>
     </row>
     <row r="78">
@@ -4679,10 +4527,8 @@
           <t>29354.66</t>
         </is>
       </c>
-      <c r="J78" s="0" t="inlineStr">
-        <is>
-          <t>416.4491</t>
-        </is>
+      <c r="J78" s="0" t="n">
+        <v>416.4491</v>
       </c>
     </row>
     <row r="79">
@@ -4726,10 +4572,8 @@
           <t>29850.95</t>
         </is>
       </c>
-      <c r="J79" s="0" t="inlineStr">
-        <is>
-          <t>418.2711</t>
-        </is>
+      <c r="J79" s="0" t="n">
+        <v>418.2711</v>
       </c>
     </row>
     <row r="80">
@@ -4773,10 +4617,8 @@
           <t>30051.71</t>
         </is>
       </c>
-      <c r="J80" s="0" t="inlineStr">
-        <is>
-          <t>418.804</t>
-        </is>
+      <c r="J80" s="0" t="n">
+        <v>418.804</v>
       </c>
     </row>
     <row r="81">
@@ -4820,10 +4662,8 @@
           <t>30163.04</t>
         </is>
       </c>
-      <c r="J81" s="0" t="inlineStr">
-        <is>
-          <t>424.1953</t>
-        </is>
+      <c r="J81" s="0" t="n">
+        <v>424.1953</v>
       </c>
     </row>
     <row r="82">
@@ -4867,10 +4707,8 @@
           <t>30162.78</t>
         </is>
       </c>
-      <c r="J82" s="0" t="inlineStr">
-        <is>
-          <t>385.3011</t>
-        </is>
+      <c r="J82" s="0" t="n">
+        <v>385.3011</v>
       </c>
     </row>
     <row r="83">
@@ -4914,10 +4752,8 @@
           <t>30102.52</t>
         </is>
       </c>
-      <c r="J83" s="0" t="inlineStr">
-        <is>
-          <t>374.979</t>
-        </is>
+      <c r="J83" s="0" t="n">
+        <v>374.979</v>
       </c>
     </row>
     <row r="84">
@@ -4961,10 +4797,8 @@
           <t>30024.57</t>
         </is>
       </c>
-      <c r="J84" s="0" t="inlineStr">
-        <is>
-          <t>385.7706</t>
-        </is>
+      <c r="J84" s="0" t="n">
+        <v>385.7706</v>
       </c>
     </row>
     <row r="85">
@@ -5008,10 +4842,8 @@
           <t>29962.89</t>
         </is>
       </c>
-      <c r="J85" s="0" t="inlineStr">
-        <is>
-          <t>371.9199</t>
-        </is>
+      <c r="J85" s="0" t="n">
+        <v>371.9199</v>
       </c>
     </row>
     <row r="86">
@@ -5055,10 +4887,8 @@
           <t>29890.58</t>
         </is>
       </c>
-      <c r="J86" s="0" t="inlineStr">
-        <is>
-          <t>388.7518</t>
-        </is>
+      <c r="J86" s="0" t="n">
+        <v>388.7518</v>
       </c>
     </row>
     <row r="87">
@@ -5102,10 +4932,8 @@
           <t>29612.95</t>
         </is>
       </c>
-      <c r="J87" s="0" t="inlineStr">
-        <is>
-          <t>395.6395</t>
-        </is>
+      <c r="J87" s="0" t="n">
+        <v>395.6395</v>
       </c>
     </row>
     <row r="88">
@@ -5149,10 +4977,8 @@
           <t>29300.37</t>
         </is>
       </c>
-      <c r="J88" s="0" t="inlineStr">
-        <is>
-          <t>395.4444</t>
-        </is>
+      <c r="J88" s="0" t="n">
+        <v>395.4444</v>
       </c>
     </row>
     <row r="89">
@@ -5196,10 +5022,8 @@
           <t>28971.8</t>
         </is>
       </c>
-      <c r="J89" s="0" t="inlineStr">
-        <is>
-          <t>383.8415</t>
-        </is>
+      <c r="J89" s="0" t="n">
+        <v>383.8415</v>
       </c>
     </row>
     <row r="90">
@@ -5243,10 +5067,8 @@
           <t>28521.5</t>
         </is>
       </c>
-      <c r="J90" s="0" t="inlineStr">
-        <is>
-          <t>340.1977</t>
-        </is>
+      <c r="J90" s="0" t="n">
+        <v>340.1977</v>
       </c>
     </row>
     <row r="91">
@@ -5290,10 +5112,8 @@
           <t>28161.38</t>
         </is>
       </c>
-      <c r="J91" s="0" t="inlineStr">
-        <is>
-          <t>321.866</t>
-        </is>
+      <c r="J91" s="0" t="n">
+        <v>321.866</v>
       </c>
     </row>
     <row r="92">
@@ -5337,10 +5157,8 @@
           <t>27792.86</t>
         </is>
       </c>
-      <c r="J92" s="0" t="inlineStr">
-        <is>
-          <t>320.5532</t>
-        </is>
+      <c r="J92" s="0" t="n">
+        <v>320.5532</v>
       </c>
     </row>
     <row r="93">
@@ -5384,10 +5202,8 @@
           <t>27484.85</t>
         </is>
       </c>
-      <c r="J93" s="0" t="inlineStr">
-        <is>
-          <t>321.3059</t>
-        </is>
+      <c r="J93" s="0" t="n">
+        <v>321.3059</v>
       </c>
     </row>
     <row r="94">
@@ -5431,10 +5247,8 @@
           <t>27247.81</t>
         </is>
       </c>
-      <c r="J94" s="0" t="inlineStr">
-        <is>
-          <t>307.9891</t>
-        </is>
+      <c r="J94" s="0" t="n">
+        <v>307.9891</v>
       </c>
     </row>
     <row r="95">
@@ -5478,10 +5292,8 @@
           <t>27043.91</t>
         </is>
       </c>
-      <c r="J95" s="0" t="inlineStr">
-        <is>
-          <t>302.8155</t>
-        </is>
+      <c r="J95" s="0" t="n">
+        <v>302.8155</v>
       </c>
     </row>
     <row r="96">
@@ -5525,10 +5337,8 @@
           <t>26890.98</t>
         </is>
       </c>
-      <c r="J96" s="0" t="inlineStr">
-        <is>
-          <t>301.0618</t>
-        </is>
+      <c r="J96" s="0" t="n">
+        <v>301.0618</v>
       </c>
     </row>
     <row r="97">
@@ -5572,10 +5382,8 @@
           <t>27012.53</t>
         </is>
       </c>
-      <c r="J97" s="0" t="inlineStr">
-        <is>
-          <t>301.8948</t>
-        </is>
+      <c r="J97" s="0" t="n">
+        <v>301.8948</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refine training validation and similarity comparisons
</commit_message>
<xml_diff>
--- a/预测文件/预测文件.xlsx
+++ b/预测文件/预测文件.xlsx
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="J2" s="0" t="n">
-        <v>342.1612</v>
+        <v>314.8961</v>
       </c>
     </row>
     <row r="3">
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="J3" s="0" t="n">
-        <v>330.3014</v>
+        <v>314.8961</v>
       </c>
     </row>
     <row r="4">
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="J4" s="0" t="n">
-        <v>324.4585</v>
+        <v>314.8961</v>
       </c>
     </row>
     <row r="5">
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="J5" s="0" t="n">
-        <v>313.4424</v>
+        <v>314.8961</v>
       </c>
     </row>
     <row r="6">
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="J6" s="0" t="n">
-        <v>300.7523</v>
+        <v>314.8961</v>
       </c>
     </row>
     <row r="7">
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="J7" s="0" t="n">
-        <v>300.7523</v>
+        <v>310.9481</v>
       </c>
     </row>
     <row r="8">
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="J8" s="0" t="n">
-        <v>300.7523</v>
+        <v>310.9481</v>
       </c>
     </row>
     <row r="9">
@@ -1450,7 +1450,7 @@
         </is>
       </c>
       <c r="J9" s="0" t="n">
-        <v>324.4585</v>
+        <v>314.8961</v>
       </c>
     </row>
     <row r="10">
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="J10" s="0" t="n">
-        <v>324.4585</v>
+        <v>314.8961</v>
       </c>
     </row>
     <row r="11">
@@ -1540,7 +1540,7 @@
         </is>
       </c>
       <c r="J11" s="0" t="n">
-        <v>313.4424</v>
+        <v>314.8961</v>
       </c>
     </row>
     <row r="12">
@@ -1585,7 +1585,7 @@
         </is>
       </c>
       <c r="J12" s="0" t="n">
-        <v>300.7523</v>
+        <v>313.0193</v>
       </c>
     </row>
     <row r="13">
@@ -1630,7 +1630,7 @@
         </is>
       </c>
       <c r="J13" s="0" t="n">
-        <v>294.0043</v>
+        <v>306.2558</v>
       </c>
     </row>
     <row r="14">
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="J14" s="0" t="n">
-        <v>288.5516</v>
+        <v>302.5071</v>
       </c>
     </row>
     <row r="15">
@@ -1720,7 +1720,7 @@
         </is>
       </c>
       <c r="J15" s="0" t="n">
-        <v>278.8357</v>
+        <v>284.2502</v>
       </c>
     </row>
     <row r="16">
@@ -1765,7 +1765,7 @@
         </is>
       </c>
       <c r="J16" s="0" t="n">
-        <v>270.8706</v>
+        <v>284.2502</v>
       </c>
     </row>
     <row r="17">
@@ -1810,7 +1810,7 @@
         </is>
       </c>
       <c r="J17" s="0" t="n">
-        <v>268.8356</v>
+        <v>283.9325</v>
       </c>
     </row>
     <row r="18">
@@ -1855,7 +1855,7 @@
         </is>
       </c>
       <c r="J18" s="0" t="n">
-        <v>268.8356</v>
+        <v>290.353</v>
       </c>
     </row>
     <row r="19">
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="J19" s="0" t="n">
-        <v>268.8356</v>
+        <v>290.353</v>
       </c>
     </row>
     <row r="20">
@@ -1945,7 +1945,7 @@
         </is>
       </c>
       <c r="J20" s="0" t="n">
-        <v>268.8356</v>
+        <v>290.353</v>
       </c>
     </row>
     <row r="21">
@@ -1990,7 +1990,7 @@
         </is>
       </c>
       <c r="J21" s="0" t="n">
-        <v>268.8356</v>
+        <v>286.047</v>
       </c>
     </row>
     <row r="22">
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="J22" s="0" t="n">
-        <v>270.4454</v>
+        <v>252.4709</v>
       </c>
     </row>
     <row r="23">
@@ -2080,7 +2080,7 @@
         </is>
       </c>
       <c r="J23" s="0" t="n">
-        <v>271.2298</v>
+        <v>252.4826</v>
       </c>
     </row>
     <row r="24">
@@ -2125,7 +2125,7 @@
         </is>
       </c>
       <c r="J24" s="0" t="n">
-        <v>271.2298</v>
+        <v>257.8509</v>
       </c>
     </row>
     <row r="25">
@@ -2170,7 +2170,7 @@
         </is>
       </c>
       <c r="J25" s="0" t="n">
-        <v>265.6194</v>
+        <v>275.2471</v>
       </c>
     </row>
     <row r="26">
@@ -2215,7 +2215,7 @@
         </is>
       </c>
       <c r="J26" s="0" t="n">
-        <v>251.6427</v>
+        <v>274.3205</v>
       </c>
     </row>
     <row r="27">
@@ -2260,7 +2260,7 @@
         </is>
       </c>
       <c r="J27" s="0" t="n">
-        <v>220.637</v>
+        <v>262.7798</v>
       </c>
     </row>
     <row r="28">
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="J28" s="0" t="n">
-        <v>210.502</v>
+        <v>237.0258</v>
       </c>
     </row>
     <row r="29">
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="J29" s="0" t="n">
-        <v>187.3375</v>
+        <v>224.4385</v>
       </c>
     </row>
     <row r="30">
@@ -2395,7 +2395,7 @@
         </is>
       </c>
       <c r="J30" s="0" t="n">
-        <v>173.0832</v>
+        <v>218.6081</v>
       </c>
     </row>
     <row r="31">
@@ -2440,7 +2440,7 @@
         </is>
       </c>
       <c r="J31" s="0" t="n">
-        <v>168.5289</v>
+        <v>204.1419</v>
       </c>
     </row>
     <row r="32">
@@ -2485,7 +2485,7 @@
         </is>
       </c>
       <c r="J32" s="0" t="n">
-        <v>150.2221</v>
+        <v>165.7043</v>
       </c>
     </row>
     <row r="33">
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="J33" s="0" t="n">
-        <v>114.1437</v>
+        <v>149.8031</v>
       </c>
     </row>
     <row r="34">
@@ -2575,7 +2575,7 @@
         </is>
       </c>
       <c r="J34" s="0" t="n">
-        <v>75.0712</v>
+        <v>106.1393</v>
       </c>
     </row>
     <row r="35">
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="J35" s="0" t="n">
-        <v>43.9015</v>
+        <v>95.79940000000001</v>
       </c>
     </row>
     <row r="36">
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="J36" s="0" t="n">
-        <v>34.6713</v>
+        <v>41.0333</v>
       </c>
     </row>
     <row r="37">
@@ -2710,7 +2710,7 @@
         </is>
       </c>
       <c r="J37" s="0" t="n">
-        <v>30.0726</v>
+        <v>32.2109</v>
       </c>
     </row>
     <row r="38">
@@ -2755,7 +2755,7 @@
         </is>
       </c>
       <c r="J38" s="0" t="n">
-        <v>28.019</v>
+        <v>24.9652</v>
       </c>
     </row>
     <row r="39">
@@ -2800,7 +2800,7 @@
         </is>
       </c>
       <c r="J39" s="0" t="n">
-        <v>27.9863</v>
+        <v>20.3666</v>
       </c>
     </row>
     <row r="40">
@@ -2845,7 +2845,7 @@
         </is>
       </c>
       <c r="J40" s="0" t="n">
-        <v>27.9863</v>
+        <v>20.048</v>
       </c>
     </row>
     <row r="41">
@@ -2890,7 +2890,7 @@
         </is>
       </c>
       <c r="J41" s="0" t="n">
-        <v>27.9863</v>
+        <v>19.5924</v>
       </c>
     </row>
     <row r="42">
@@ -2935,7 +2935,7 @@
         </is>
       </c>
       <c r="J42" s="0" t="n">
-        <v>4.4122</v>
+        <v>17.8908</v>
       </c>
     </row>
     <row r="43">
@@ -2980,7 +2980,7 @@
         </is>
       </c>
       <c r="J43" s="0" t="n">
-        <v>4.4122</v>
+        <v>17.8908</v>
       </c>
     </row>
     <row r="44">
@@ -3025,7 +3025,7 @@
         </is>
       </c>
       <c r="J44" s="0" t="n">
-        <v>4.6512</v>
+        <v>17.8908</v>
       </c>
     </row>
     <row r="45">
@@ -3070,7 +3070,7 @@
         </is>
       </c>
       <c r="J45" s="0" t="n">
-        <v>4.7505</v>
+        <v>17.8908</v>
       </c>
     </row>
     <row r="46">
@@ -3115,7 +3115,7 @@
         </is>
       </c>
       <c r="J46" s="0" t="n">
-        <v>4.1659</v>
+        <v>17.0499</v>
       </c>
     </row>
     <row r="47">
@@ -3160,7 +3160,7 @@
         </is>
       </c>
       <c r="J47" s="0" t="n">
-        <v>4.1755</v>
+        <v>17.0499</v>
       </c>
     </row>
     <row r="48">
@@ -3205,7 +3205,7 @@
         </is>
       </c>
       <c r="J48" s="0" t="n">
-        <v>4.1904</v>
+        <v>17.0499</v>
       </c>
     </row>
     <row r="49">
@@ -3250,7 +3250,7 @@
         </is>
       </c>
       <c r="J49" s="0" t="n">
-        <v>4.1904</v>
+        <v>17.0499</v>
       </c>
     </row>
     <row r="50">
@@ -3295,7 +3295,7 @@
         </is>
       </c>
       <c r="J50" s="0" t="n">
-        <v>4.097</v>
+        <v>16.812</v>
       </c>
     </row>
     <row r="51">
@@ -3340,7 +3340,7 @@
         </is>
       </c>
       <c r="J51" s="0" t="n">
-        <v>4.1476</v>
+        <v>16.812</v>
       </c>
     </row>
     <row r="52">
@@ -3385,7 +3385,7 @@
         </is>
       </c>
       <c r="J52" s="0" t="n">
-        <v>4.2242</v>
+        <v>16.8595</v>
       </c>
     </row>
     <row r="53">
@@ -3430,7 +3430,7 @@
         </is>
       </c>
       <c r="J53" s="0" t="n">
-        <v>4.4815</v>
+        <v>17.1399</v>
       </c>
     </row>
     <row r="54">
@@ -3475,7 +3475,7 @@
         </is>
       </c>
       <c r="J54" s="0" t="n">
-        <v>4.9529</v>
+        <v>17.8146</v>
       </c>
     </row>
     <row r="55">
@@ -3520,7 +3520,7 @@
         </is>
       </c>
       <c r="J55" s="0" t="n">
-        <v>4.9529</v>
+        <v>17.8146</v>
       </c>
     </row>
     <row r="56">
@@ -3565,7 +3565,7 @@
         </is>
       </c>
       <c r="J56" s="0" t="n">
-        <v>4.9529</v>
+        <v>17.6891</v>
       </c>
     </row>
     <row r="57">
@@ -3610,7 +3610,7 @@
         </is>
       </c>
       <c r="J57" s="0" t="n">
-        <v>5.4199</v>
+        <v>18.3169</v>
       </c>
     </row>
     <row r="58">
@@ -3655,7 +3655,7 @@
         </is>
       </c>
       <c r="J58" s="0" t="n">
-        <v>6.0135</v>
+        <v>19.4072</v>
       </c>
     </row>
     <row r="59">
@@ -3700,7 +3700,7 @@
         </is>
       </c>
       <c r="J59" s="0" t="n">
-        <v>5.8903</v>
+        <v>19.4072</v>
       </c>
     </row>
     <row r="60">
@@ -3745,7 +3745,7 @@
         </is>
       </c>
       <c r="J60" s="0" t="n">
-        <v>5.9955</v>
+        <v>19.4072</v>
       </c>
     </row>
     <row r="61">
@@ -3790,7 +3790,7 @@
         </is>
       </c>
       <c r="J61" s="0" t="n">
-        <v>5.9669</v>
+        <v>19.7961</v>
       </c>
     </row>
     <row r="62">
@@ -3835,7 +3835,7 @@
         </is>
       </c>
       <c r="J62" s="0" t="n">
-        <v>62.9526</v>
+        <v>20.3585</v>
       </c>
     </row>
     <row r="63">
@@ -3880,7 +3880,7 @@
         </is>
       </c>
       <c r="J63" s="0" t="n">
-        <v>62.9526</v>
+        <v>20.3585</v>
       </c>
     </row>
     <row r="64">
@@ -3925,7 +3925,7 @@
         </is>
       </c>
       <c r="J64" s="0" t="n">
-        <v>62.9313</v>
+        <v>21.3809</v>
       </c>
     </row>
     <row r="65">
@@ -3970,7 +3970,7 @@
         </is>
       </c>
       <c r="J65" s="0" t="n">
-        <v>62.9313</v>
+        <v>25.9795</v>
       </c>
     </row>
     <row r="66">
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="J66" s="0" t="n">
-        <v>64.7629</v>
+        <v>26.8458</v>
       </c>
     </row>
     <row r="67">
@@ -4060,7 +4060,7 @@
         </is>
       </c>
       <c r="J67" s="0" t="n">
-        <v>79.9581</v>
+        <v>42.9139</v>
       </c>
     </row>
     <row r="68">
@@ -4105,7 +4105,7 @@
         </is>
       </c>
       <c r="J68" s="0" t="n">
-        <v>86.79900000000001</v>
+        <v>198.9137</v>
       </c>
     </row>
     <row r="69">
@@ -4150,7 +4150,7 @@
         </is>
       </c>
       <c r="J69" s="0" t="n">
-        <v>120.9955</v>
+        <v>210.3134</v>
       </c>
     </row>
     <row r="70">
@@ -4195,7 +4195,7 @@
         </is>
       </c>
       <c r="J70" s="0" t="n">
-        <v>164.9454</v>
+        <v>213.548</v>
       </c>
     </row>
     <row r="71">
@@ -4240,7 +4240,7 @@
         </is>
       </c>
       <c r="J71" s="0" t="n">
-        <v>191.7761</v>
+        <v>230.9196</v>
       </c>
     </row>
     <row r="72">
@@ -4285,7 +4285,7 @@
         </is>
       </c>
       <c r="J72" s="0" t="n">
-        <v>224.4741</v>
+        <v>245.7555</v>
       </c>
     </row>
     <row r="73">
@@ -4330,7 +4330,7 @@
         </is>
       </c>
       <c r="J73" s="0" t="n">
-        <v>245.4175</v>
+        <v>260.4942</v>
       </c>
     </row>
     <row r="74">
@@ -4375,7 +4375,7 @@
         </is>
       </c>
       <c r="J74" s="0" t="n">
-        <v>262.9271</v>
+        <v>360.9023</v>
       </c>
     </row>
     <row r="75">
@@ -4420,7 +4420,7 @@
         </is>
       </c>
       <c r="J75" s="0" t="n">
-        <v>298.582</v>
+        <v>360.9023</v>
       </c>
     </row>
     <row r="76">
@@ -4465,7 +4465,7 @@
         </is>
       </c>
       <c r="J76" s="0" t="n">
-        <v>307.8188</v>
+        <v>360.9023</v>
       </c>
     </row>
     <row r="77">
@@ -4510,7 +4510,7 @@
         </is>
       </c>
       <c r="J77" s="0" t="n">
-        <v>311.5489</v>
+        <v>360.9023</v>
       </c>
     </row>
     <row r="78">
@@ -4555,7 +4555,7 @@
         </is>
       </c>
       <c r="J78" s="0" t="n">
-        <v>311.4686</v>
+        <v>359.882</v>
       </c>
     </row>
     <row r="79">
@@ -4600,7 +4600,7 @@
         </is>
       </c>
       <c r="J79" s="0" t="n">
-        <v>315.9866</v>
+        <v>359.882</v>
       </c>
     </row>
     <row r="80">
@@ -4645,7 +4645,7 @@
         </is>
       </c>
       <c r="J80" s="0" t="n">
-        <v>318.5092</v>
+        <v>366.8422</v>
       </c>
     </row>
     <row r="81">
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="J81" s="0" t="n">
-        <v>312.8808</v>
+        <v>359.882</v>
       </c>
     </row>
     <row r="82">
@@ -4735,7 +4735,7 @@
         </is>
       </c>
       <c r="J82" s="0" t="n">
-        <v>311.1101</v>
+        <v>359.9656</v>
       </c>
     </row>
     <row r="83">
@@ -4780,7 +4780,7 @@
         </is>
       </c>
       <c r="J83" s="0" t="n">
-        <v>305.2048</v>
+        <v>359.9656</v>
       </c>
     </row>
     <row r="84">
@@ -4825,7 +4825,7 @@
         </is>
       </c>
       <c r="J84" s="0" t="n">
-        <v>304.3397</v>
+        <v>359.7922</v>
       </c>
     </row>
     <row r="85">
@@ -4870,7 +4870,7 @@
         </is>
       </c>
       <c r="J85" s="0" t="n">
-        <v>302.3256</v>
+        <v>360.636</v>
       </c>
     </row>
     <row r="86">
@@ -4915,7 +4915,7 @@
         </is>
       </c>
       <c r="J86" s="0" t="n">
-        <v>300.5637</v>
+        <v>360.1993</v>
       </c>
     </row>
     <row r="87">
@@ -4960,7 +4960,7 @@
         </is>
       </c>
       <c r="J87" s="0" t="n">
-        <v>300.5637</v>
+        <v>361.2597</v>
       </c>
     </row>
     <row r="88">
@@ -5005,7 +5005,7 @@
         </is>
       </c>
       <c r="J88" s="0" t="n">
-        <v>299.2323</v>
+        <v>318.927</v>
       </c>
     </row>
     <row r="89">
@@ -5050,7 +5050,7 @@
         </is>
       </c>
       <c r="J89" s="0" t="n">
-        <v>294.7225</v>
+        <v>318.927</v>
       </c>
     </row>
     <row r="90">
@@ -5095,7 +5095,7 @@
         </is>
       </c>
       <c r="J90" s="0" t="n">
-        <v>296.2437</v>
+        <v>318.927</v>
       </c>
     </row>
     <row r="91">
@@ -5140,7 +5140,7 @@
         </is>
       </c>
       <c r="J91" s="0" t="n">
-        <v>290.0397</v>
+        <v>318.927</v>
       </c>
     </row>
     <row r="92">
@@ -5185,7 +5185,7 @@
         </is>
       </c>
       <c r="J92" s="0" t="n">
-        <v>287.6973</v>
+        <v>318.2673</v>
       </c>
     </row>
     <row r="93">
@@ -5230,7 +5230,7 @@
         </is>
       </c>
       <c r="J93" s="0" t="n">
-        <v>286.1994</v>
+        <v>319.884</v>
       </c>
     </row>
     <row r="94">
@@ -5275,7 +5275,7 @@
         </is>
       </c>
       <c r="J94" s="0" t="n">
-        <v>286.1994</v>
+        <v>318.1001</v>
       </c>
     </row>
     <row r="95">
@@ -5320,7 +5320,7 @@
         </is>
       </c>
       <c r="J95" s="0" t="n">
-        <v>286.1994</v>
+        <v>318.1001</v>
       </c>
     </row>
     <row r="96">
@@ -5365,7 +5365,7 @@
         </is>
       </c>
       <c r="J96" s="0" t="n">
-        <v>286.1994</v>
+        <v>318.1001</v>
       </c>
     </row>
     <row r="97">
@@ -5410,7 +5410,7 @@
         </is>
       </c>
       <c r="J97" s="0" t="n">
-        <v>286.1994</v>
+        <v>318.1001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update price model training and prediction workflows
</commit_message>
<xml_diff>
--- a/预测文件/预测文件.xlsx
+++ b/预测文件/预测文件.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowHeight="16155" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="26880" windowHeight="17595" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1030,7 +1030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J97"/>
+  <dimension ref="A1:I97"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="18.25" customWidth="1" style="1" min="2" max="9"/>
@@ -1044,47 +1044,42 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>5.11日风光电力值(MW)</t>
+          <t>5.28日风光电力值(MW)</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>5.11日总加电力值(MW)</t>
+          <t>5.28日总加电力值(MW)</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>5.11日剩余电力值</t>
+          <t>5.28日剩余电力值</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>5.11日日前出清价格(元/MWh)</t>
+          <t>5.28日日前出清价格(元/MWh)</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>5.12日风光电力值(MW)</t>
+          <t>5.29日风光电力值(MW)</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>5.12日总加电力值(MW)</t>
+          <t>5.29日总加电力值(MW)</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>5.12日剩余电力值</t>
+          <t>5.29日剩余电力值</t>
         </is>
       </c>
       <c r="I1" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">火电开机容量 </t>
-        </is>
-      </c>
-      <c r="J1" s="0" t="inlineStr">
-        <is>
-          <t>预测价格</t>
         </is>
       </c>
     </row>
@@ -1096,46 +1091,43 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>3363.85</t>
+          <t>13986.97</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
         <is>
-          <t>35636.5</t>
+          <t>32687.3</t>
         </is>
       </c>
       <c r="D2" s="0" t="inlineStr">
         <is>
-          <t>32272.65</t>
+          <t>18700.33</t>
         </is>
       </c>
       <c r="E2" s="0" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>275</t>
         </is>
       </c>
       <c r="F2" s="0" t="inlineStr">
         <is>
-          <t>8340.11</t>
+          <t>2738.62</t>
         </is>
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t>34906.1</t>
+          <t>32835.6</t>
         </is>
       </c>
       <c r="H2" s="0" t="inlineStr">
         <is>
-          <t>26565.99</t>
+          <t>30096.98</t>
         </is>
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
-          <t>33225</t>
-        </is>
-      </c>
-      <c r="J2" s="0" t="n">
-        <v>315.0613</v>
+          <t>38075</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -1146,41 +1138,38 @@
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>3215</t>
+          <t>13928.7</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>35502.7</t>
+          <t>32201.3</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>32287.7</t>
+          <t>18272.6</t>
         </is>
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
-          <t>567</t>
+          <t>275</t>
         </is>
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>8349.11</t>
+          <t>2657.43</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>34647.8</t>
+          <t>32540.6</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
         <is>
-          <t>26298.69</t>
-        </is>
-      </c>
-      <c r="J3" s="0" t="n">
-        <v>309.0041</v>
+          <t>29883.17</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -1191,41 +1180,38 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>3069.46</t>
+          <t>13875.19</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>35434.1</t>
+          <t>31971.9</t>
         </is>
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>32364.64</t>
+          <t>18096.71</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>564</t>
+          <t>281</t>
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>8351.58</t>
+          <t>2582.64</t>
         </is>
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>34422.6</t>
+          <t>32270.6</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
         <is>
-          <t>26071.02</t>
-        </is>
-      </c>
-      <c r="J4" s="0" t="n">
-        <v>307.2555</v>
+          <t>29687.96</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -1236,41 +1222,38 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>2943.09</t>
+          <t>13815.2</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>35332.8</t>
+          <t>31673.1</t>
         </is>
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t>32389.71</t>
+          <t>17857.9</t>
         </is>
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>564</t>
+          <t>269</t>
         </is>
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t>8347.82</t>
+          <t>2505.69</t>
         </is>
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>34236.6</t>
+          <t>31999.6</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t>25888.78</t>
-        </is>
-      </c>
-      <c r="J5" s="0" t="n">
-        <v>307.2555</v>
+          <t>29493.91</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -1281,41 +1264,38 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>2836.78</t>
+          <t>13761.58</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>35088.4</t>
+          <t>31559.4</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>32251.62</t>
+          <t>17797.82</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>269</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>8313.1</t>
+          <t>2446.77</t>
         </is>
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>33971.2</t>
+          <t>31797.6</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
-          <t>25658.1</t>
-        </is>
-      </c>
-      <c r="J6" s="0" t="n">
-        <v>307.2555</v>
+          <t>29350.83</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -1326,41 +1306,38 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>2732.5</t>
+          <t>13716.1</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>34814</t>
+          <t>31440.5</t>
         </is>
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>32081.5</t>
+          <t>17724.4</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>455</t>
+          <t>259.1</t>
         </is>
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>8268.54</t>
+          <t>2398.49</t>
         </is>
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>33787.4</t>
+          <t>31590.6</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t>25518.86</t>
-        </is>
-      </c>
-      <c r="J7" s="0" t="n">
-        <v>307.2555</v>
+          <t>29192.11</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -1371,41 +1348,38 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>2637.47</t>
+          <t>13681.27</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>34399.4</t>
+          <t>31322.7</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>31761.93</t>
+          <t>17641.43</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>459</t>
+          <t>269</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>8224.03</t>
+          <t>2351.84</t>
         </is>
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>33675.8</t>
+          <t>31567.8</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t>25451.77</t>
-        </is>
-      </c>
-      <c r="J8" s="0" t="n">
-        <v>307.2555</v>
+          <t>29215.96</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -1416,41 +1390,38 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>2552.14</t>
+          <t>13639.15</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>34469.5</t>
+          <t>31297.4</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>31917.36</t>
+          <t>17658.25</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t>453</t>
+          <t>260</t>
         </is>
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>8168.69</t>
+          <t>2315.78</t>
         </is>
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>34643.3</t>
+          <t>31682</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t>26474.61</t>
-        </is>
-      </c>
-      <c r="J9" s="0" t="n">
-        <v>307.2555</v>
+          <t>29366.22</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1461,41 +1432,38 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>2470.88</t>
+          <t>13623.91</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>35576.2</t>
+          <t>31831.5</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>33105.32</t>
+          <t>18207.59</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>917</t>
+          <t>271</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>8100.61</t>
+          <t>2289.78</t>
         </is>
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>34830.1</t>
+          <t>32451.6</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
-          <t>26729.49</t>
-        </is>
-      </c>
-      <c r="J10" s="0" t="n">
-        <v>313.3127</v>
+          <t>30161.82</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -1506,41 +1474,38 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>2391.6</t>
+          <t>13614.96</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>35327.8</t>
+          <t>31879.8</t>
         </is>
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t>32936.2</t>
+          <t>18264.84</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>580</t>
+          <t>260</t>
         </is>
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t>8022.18</t>
+          <t>2272.59</t>
         </is>
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>34491.8</t>
+          <t>32476.6</t>
         </is>
       </c>
       <c r="H11" s="0" t="inlineStr">
         <is>
-          <t>26469.62</t>
-        </is>
-      </c>
-      <c r="J11" s="0" t="n">
-        <v>307.2555</v>
+          <t>30204.01</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1551,41 +1516,38 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>2312.19</t>
+          <t>13606.82</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>34764.5</t>
+          <t>31720.8</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t>32452.31</t>
+          <t>18113.98</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>800</t>
+          <t>273</t>
         </is>
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>7941.68</t>
+          <t>2266.07</t>
         </is>
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>34186.6</t>
+          <t>32252.6</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
-          <t>26244.92</t>
-        </is>
-      </c>
-      <c r="J12" s="0" t="n">
-        <v>307.2555</v>
+          <t>29986.53</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -1596,41 +1558,38 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>2234.14</t>
+          <t>13596.26</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t>34652.4</t>
+          <t>31514.5</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>32418.26</t>
+          <t>17918.24</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t>800</t>
+          <t>260</t>
         </is>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>7848.41</t>
+          <t>2253.24</t>
         </is>
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>33883.4</t>
+          <t>32027.6</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t>26034.99</t>
-        </is>
-      </c>
-      <c r="J13" s="0" t="n">
-        <v>307.2555</v>
+          <t>29774.36</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -1641,41 +1600,38 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>2166.33</t>
+          <t>13599.13</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t>34535.3</t>
+          <t>31333.4</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t>32368.97</t>
+          <t>17734.27</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t>575</t>
+          <t>257</t>
         </is>
       </c>
       <c r="F14" s="0" t="inlineStr">
         <is>
-          <t>7757.44</t>
+          <t>2249.25</t>
         </is>
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>33761</t>
+          <t>31804.6</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
         <is>
-          <t>26003.56</t>
-        </is>
-      </c>
-      <c r="J14" s="0" t="n">
-        <v>307.2555</v>
+          <t>29555.35</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -1686,41 +1642,38 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>2105.7</t>
+          <t>13607.78</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t>34518.7</t>
+          <t>31193.6</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t>32413</t>
+          <t>17585.82</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>580</t>
+          <t>260</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t>7655.85</t>
+          <t>2254.18</t>
         </is>
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>33736.5</t>
+          <t>31599.6</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
         <is>
-          <t>26080.65</t>
-        </is>
-      </c>
-      <c r="J15" s="0" t="n">
-        <v>307.2555</v>
+          <t>29345.42</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -1731,41 +1684,38 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>2050.9</t>
+          <t>13610.54</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>34185</t>
+          <t>31240.8</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>32134.1</t>
+          <t>17630.26</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>260</t>
         </is>
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>7562.92</t>
+          <t>2257.9</t>
         </is>
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>33743.2</t>
+          <t>31260.6</t>
         </is>
       </c>
       <c r="H16" s="0" t="inlineStr">
         <is>
-          <t>26180.28</t>
-        </is>
-      </c>
-      <c r="J16" s="0" t="n">
-        <v>307.2555</v>
+          <t>29002.7</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -1776,41 +1726,38 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>1999.36</t>
+          <t>13608.49</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>34094.3</t>
+          <t>30963.1</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t>32094.94</t>
+          <t>17354.61</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>564</t>
+          <t>260</t>
         </is>
       </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
-          <t>7466.83</t>
+          <t>2255.75</t>
         </is>
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>33639.3</t>
+          <t>31123.6</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
         <is>
-          <t>26172.47</t>
-        </is>
-      </c>
-      <c r="J17" s="0" t="n">
-        <v>307.2555</v>
+          <t>28867.85</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -1821,41 +1768,38 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>1968.2</t>
+          <t>13592.47</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>34067.6</t>
+          <t>31126.1</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t>32099.4</t>
+          <t>17533.63</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>564</t>
+          <t>260</t>
         </is>
       </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
-          <t>7384.57</t>
+          <t>2251.73</t>
         </is>
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>33716.3</t>
+          <t>31124.6</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t>26331.73</t>
-        </is>
-      </c>
-      <c r="J18" s="0" t="n">
-        <v>307.2555</v>
+          <t>28872.87</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -1866,41 +1810,38 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>1946.57</t>
+          <t>13560.28</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>34265.4</t>
+          <t>31070.8</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>32318.83</t>
+          <t>17510.52</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>567</t>
+          <t>260</t>
         </is>
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>7304.58</t>
+          <t>2250.21</t>
         </is>
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>33592.7</t>
+          <t>31138.6</t>
         </is>
       </c>
       <c r="H19" s="0" t="inlineStr">
         <is>
-          <t>26288.12</t>
-        </is>
-      </c>
-      <c r="J19" s="0" t="n">
-        <v>307.2555</v>
+          <t>28888.39</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1911,41 +1852,38 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>1924.92</t>
+          <t>13528.5</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>33980.5</t>
+          <t>31041.7</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t>32055.58</t>
+          <t>17513.2</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>569</t>
+          <t>260</t>
         </is>
       </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
-          <t>7227.87</t>
+          <t>2245.32</t>
         </is>
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>33475.3</t>
+          <t>31178.6</t>
         </is>
       </c>
       <c r="H20" s="0" t="inlineStr">
         <is>
-          <t>26247.43</t>
-        </is>
-      </c>
-      <c r="J20" s="0" t="n">
-        <v>307.2555</v>
+          <t>28933.28</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -1956,41 +1894,38 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>1900.22</t>
+          <t>13486.3</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t>33900.9</t>
+          <t>31033.7</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t>32000.68</t>
+          <t>17547.4</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>564</t>
+          <t>260</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>7147.74</t>
+          <t>2243.49</t>
         </is>
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>33430.3</t>
+          <t>31192.6</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
         <is>
-          <t>26282.56</t>
-        </is>
-      </c>
-      <c r="J21" s="0" t="n">
-        <v>307.2555</v>
+          <t>28949.11</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -2001,41 +1936,38 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>1874.43</t>
+          <t>13437.26</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>34035.7</t>
+          <t>31028.7</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>32161.27</t>
+          <t>17591.44</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>260</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>7069.77</t>
+          <t>2271.34</t>
         </is>
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>33652.5</t>
+          <t>31364.7</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
         <is>
-          <t>26582.73</t>
-        </is>
-      </c>
-      <c r="J22" s="0" t="n">
-        <v>312.1381</v>
+          <t>29093.36</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -2046,41 +1978,38 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>1890.12</t>
+          <t>13494.72</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>34496.2</t>
+          <t>31372.7</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t>32606.08</t>
+          <t>17877.98</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>275</t>
         </is>
       </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
-          <t>7055.32</t>
+          <t>2409.09</t>
         </is>
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>33990.5</t>
+          <t>31666.9</t>
         </is>
       </c>
       <c r="H23" s="0" t="inlineStr">
         <is>
-          <t>26935.18</t>
-        </is>
-      </c>
-      <c r="J23" s="0" t="n">
-        <v>312.1381</v>
+          <t>29257.81</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -2091,41 +2020,38 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>2030.93</t>
+          <t>13700.75</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>34789</t>
+          <t>31685</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t>32758.07</t>
+          <t>17984.25</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>920</t>
+          <t>269</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>7158.86</t>
+          <t>2724.92</t>
         </is>
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>34259.2</t>
+          <t>32226.6</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
         <is>
-          <t>27100.34</t>
-        </is>
-      </c>
-      <c r="J24" s="0" t="n">
-        <v>311.1047</v>
+          <t>29501.68</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -2136,41 +2062,38 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>2391.99</t>
+          <t>14101.66</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>34844</t>
+          <t>31746.1</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>32452.01</t>
+          <t>17644.44</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>917</t>
+          <t>259.99</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>7466.97</t>
+          <t>3248.12</t>
         </is>
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>34351.4</t>
+          <t>32544.8</t>
         </is>
       </c>
       <c r="H25" s="0" t="inlineStr">
         <is>
-          <t>26884.43</t>
-        </is>
-      </c>
-      <c r="J25" s="0" t="n">
-        <v>311.1047</v>
+          <t>29296.68</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -2181,41 +2104,38 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>3014.14</t>
+          <t>14619.63</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t>34879</t>
+          <t>31936.2</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>31864.86</t>
+          <t>17316.57</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>290.67</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>8013.33</t>
+          <t>3941.53</t>
         </is>
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>34720.9</t>
+          <t>32732.8</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
         <is>
-          <t>26707.57</t>
-        </is>
-      </c>
-      <c r="J26" s="0" t="n">
-        <v>311.1047</v>
+          <t>28791.27</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -2226,41 +2146,38 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>3823.18</t>
+          <t>15264.57</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t>34794.2</t>
+          <t>31679.2</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>30971.02</t>
+          <t>16414.63</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>456</t>
+          <t>254</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>8733.16</t>
+          <t>4788.67</t>
         </is>
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>34585.9</t>
+          <t>32532.4</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
         <is>
-          <t>25852.74</t>
-        </is>
-      </c>
-      <c r="J27" s="0" t="n">
-        <v>307.2555</v>
+          <t>27743.73</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -2271,41 +2188,38 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>4773.72</t>
+          <t>15982.16</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t>34227.7</t>
+          <t>31351.7</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>29453.98</t>
+          <t>15369.54</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>240</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>9572.56</t>
+          <t>5740.75</t>
         </is>
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>34229.8</t>
+          <t>32118.4</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
         <is>
-          <t>24657.24</t>
-        </is>
-      </c>
-      <c r="J28" s="0" t="n">
-        <v>307.2555</v>
+          <t>26377.65</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -2316,41 +2230,38 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>5911.3</t>
+          <t>16823.14</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t>33852.1</t>
+          <t>30178.3</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>27940.8</t>
+          <t>13355.16</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>10597.09</t>
+          <t>6852.74</t>
         </is>
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>33785.6</t>
+          <t>31902.5</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
         <is>
-          <t>23188.51</t>
-        </is>
-      </c>
-      <c r="J29" s="0" t="n">
-        <v>307.2555</v>
+          <t>25049.76</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -2361,41 +2272,38 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>7136.15</t>
+          <t>17715.29</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t>33398.4</t>
+          <t>29605.5</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t>26262.25</t>
+          <t>11890.21</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>299</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t>11686.54</t>
+          <t>8004.96</t>
         </is>
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>33332.4</t>
+          <t>31639.5</t>
         </is>
       </c>
       <c r="H30" s="0" t="inlineStr">
         <is>
-          <t>21645.86</t>
-        </is>
-      </c>
-      <c r="J30" s="0" t="n">
-        <v>300.5916</v>
+          <t>23634.54</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -2406,41 +2314,38 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>8496.27</t>
+          <t>18681.82</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>33042.3</t>
+          <t>29587.5</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t>24546.03</t>
+          <t>10905.68</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>284</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
         <is>
-          <t>12896.65</t>
+          <t>9256.49</t>
         </is>
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>32961.2</t>
+          <t>31504.6</t>
         </is>
       </c>
       <c r="H31" s="0" t="inlineStr">
         <is>
-          <t>20064.55</t>
-        </is>
-      </c>
-      <c r="J31" s="0" t="n">
-        <v>283.1887</v>
+          <t>22248.11</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -2451,41 +2356,38 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>9965.86</t>
+          <t>19704.13</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>32797.9</t>
+          <t>29675.7</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t>22832.04</t>
+          <t>9971.57</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t>272</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t>14195</t>
+          <t>10584.32</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>32709.5</t>
+          <t>31246.7</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
         <is>
-          <t>18514.5</t>
-        </is>
-      </c>
-      <c r="J32" s="0" t="n">
-        <v>282.7488</v>
+          <t>20662.38</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -2496,41 +2398,38 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>11423.38</t>
+          <t>20578.97</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>32401.8</t>
+          <t>29862.3</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t>20978.42</t>
+          <t>9283.33</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t>268</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t>15463.16</t>
+          <t>11830.84</t>
         </is>
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>32261.1</t>
+          <t>30824.5</t>
         </is>
       </c>
       <c r="H33" s="0" t="inlineStr">
         <is>
-          <t>16797.94</t>
-        </is>
-      </c>
-      <c r="J33" s="0" t="n">
-        <v>270.7629</v>
+          <t>18993.66</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -2541,41 +2440,38 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>12943.94</t>
+          <t>21603.28</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t>32049.3</t>
+          <t>30883.6</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>19105.36</t>
+          <t>9280.32</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t>267</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F34" s="0" t="inlineStr">
         <is>
-          <t>16846.39</t>
+          <t>13181.29</t>
         </is>
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>32081.9</t>
+          <t>30983</t>
         </is>
       </c>
       <c r="H34" s="0" t="inlineStr">
         <is>
-          <t>15235.51</t>
-        </is>
-      </c>
-      <c r="J34" s="0" t="n">
-        <v>138.5679</v>
+          <t>17801.71</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -2586,41 +2482,38 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>14473.31</t>
+          <t>22610.68</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t>31444.7</t>
+          <t>30910.1</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t>16971.39</t>
+          <t>8299.42</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F35" s="0" t="inlineStr">
         <is>
-          <t>18232.71</t>
+          <t>14516.2</t>
         </is>
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>31942.7</t>
+          <t>30500</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
         <is>
-          <t>13709.99</t>
-        </is>
-      </c>
-      <c r="J35" s="0" t="n">
-        <v>142.7832</v>
+          <t>15983.8</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -2631,17 +2524,17 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>15950.29</t>
+          <t>23582.98</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t>31152</t>
+          <t>30694.3</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t>15201.71</t>
+          <t>7111.32</t>
         </is>
       </c>
       <c r="E36" s="0" t="inlineStr">
@@ -2651,21 +2544,18 @@
       </c>
       <c r="F36" s="0" t="inlineStr">
         <is>
-          <t>19580.22</t>
+          <t>15815.93</t>
         </is>
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>31655.8</t>
+          <t>30240.5</t>
         </is>
       </c>
       <c r="H36" s="0" t="inlineStr">
         <is>
-          <t>12075.58</t>
-        </is>
-      </c>
-      <c r="J36" s="0" t="n">
-        <v>59.3528</v>
+          <t>14424.57</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -2676,17 +2566,17 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>17281.71</t>
+          <t>24381.48</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t>31826.9</t>
+          <t>30995.8</t>
         </is>
       </c>
       <c r="D37" s="0" t="inlineStr">
         <is>
-          <t>14545.19</t>
+          <t>6614.32</t>
         </is>
       </c>
       <c r="E37" s="0" t="inlineStr">
@@ -2696,21 +2586,18 @@
       </c>
       <c r="F37" s="0" t="inlineStr">
         <is>
-          <t>20798.9</t>
+          <t>16979.85</t>
         </is>
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>31963.7</t>
+          <t>30629.5</t>
         </is>
       </c>
       <c r="H37" s="0" t="inlineStr">
         <is>
-          <t>11164.8</t>
-        </is>
-      </c>
-      <c r="J37" s="0" t="n">
-        <v>48.4298</v>
+          <t>13649.65</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -2721,17 +2608,17 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>18578.09</t>
+          <t>25191</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t>32436.6</t>
+          <t>31196.6</t>
         </is>
       </c>
       <c r="D38" s="0" t="inlineStr">
         <is>
-          <t>13858.51</t>
+          <t>6005.6</t>
         </is>
       </c>
       <c r="E38" s="0" t="inlineStr">
@@ -2741,21 +2628,18 @@
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>22068.66</t>
+          <t>18168.4</t>
         </is>
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>32424.2</t>
+          <t>30819.6</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
         <is>
-          <t>10355.54</t>
-        </is>
-      </c>
-      <c r="J38" s="0" t="n">
-        <v>78.7212</v>
+          <t>12651.2</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -2766,17 +2650,17 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>19782.73</t>
+          <t>25897.39</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t>31968</t>
+          <t>31139.1</t>
         </is>
       </c>
       <c r="D39" s="0" t="inlineStr">
         <is>
-          <t>12185.27</t>
+          <t>5241.71</t>
         </is>
       </c>
       <c r="E39" s="0" t="inlineStr">
@@ -2786,21 +2670,18 @@
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>23285.52</t>
+          <t>19293.52</t>
         </is>
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>31998.5</t>
+          <t>30619.1</t>
         </is>
       </c>
       <c r="H39" s="0" t="inlineStr">
         <is>
-          <t>8712.98</t>
-        </is>
-      </c>
-      <c r="J39" s="0" t="n">
-        <v>19.0374</v>
+          <t>11325.58</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -2811,17 +2692,17 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>20876.04</t>
+          <t>26601.59</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t>31690.6</t>
+          <t>30908.9</t>
         </is>
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>10814.56</t>
+          <t>4307.31</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
@@ -2831,21 +2712,18 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>24408.4</t>
+          <t>20348.01</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>31551.4</t>
+          <t>30474</t>
         </is>
       </c>
       <c r="H40" s="0" t="inlineStr">
         <is>
-          <t>7143</t>
-        </is>
-      </c>
-      <c r="J40" s="0" t="n">
-        <v>14.4676</v>
+          <t>10125.99</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -2856,17 +2734,17 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>21831.44</t>
+          <t>27176.61</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
-          <t>31245.9</t>
+          <t>30652.9</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t>9414.46</t>
+          <t>3476.29</t>
         </is>
       </c>
       <c r="E41" s="0" t="inlineStr">
@@ -2876,21 +2754,18 @@
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>25404.33</t>
+          <t>21291.71</t>
         </is>
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>31298.4</t>
+          <t>30273.5</t>
         </is>
       </c>
       <c r="H41" s="0" t="inlineStr">
         <is>
-          <t>5894.07</t>
-        </is>
-      </c>
-      <c r="J41" s="0" t="n">
-        <v>14.4676</v>
+          <t>8981.79</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -2901,17 +2776,17 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>22710.61</t>
+          <t>27709.4</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
-          <t>31054.6</t>
+          <t>30528.9</t>
         </is>
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>8343.99</t>
+          <t>2819.5</t>
         </is>
       </c>
       <c r="E42" s="0" t="inlineStr">
@@ -2921,21 +2796,18 @@
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>26349.45</t>
+          <t>22149.06</t>
         </is>
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>31277.3</t>
+          <t>29972.2</t>
         </is>
       </c>
       <c r="H42" s="0" t="inlineStr">
         <is>
-          <t>4927.85</t>
-        </is>
-      </c>
-      <c r="J42" s="0" t="n">
-        <v>14.4676</v>
+          <t>7823.14</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -2946,17 +2818,17 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>23494.87</t>
+          <t>28150.28</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
-          <t>30860.4</t>
+          <t>30310.8</t>
         </is>
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>7365.53</t>
+          <t>2160.52</t>
         </is>
       </c>
       <c r="E43" s="0" t="inlineStr">
@@ -2966,21 +2838,18 @@
       </c>
       <c r="F43" s="0" t="inlineStr">
         <is>
-          <t>27191.48</t>
+          <t>22920.71</t>
         </is>
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>31146.9</t>
+          <t>29674.8</t>
         </is>
       </c>
       <c r="H43" s="0" t="inlineStr">
         <is>
-          <t>3955.42</t>
-        </is>
-      </c>
-      <c r="J43" s="0" t="n">
-        <v>13.2787</v>
+          <t>6754.09</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -2991,17 +2860,17 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>24162.7</t>
+          <t>28542.73</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
         <is>
-          <t>30757.4</t>
+          <t>29995.3</t>
         </is>
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>6594.7</t>
+          <t>1452.57</t>
         </is>
       </c>
       <c r="E44" s="0" t="inlineStr">
@@ -3011,21 +2880,18 @@
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>27934.05</t>
+          <t>23615.26</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>31006.7</t>
+          <t>29569.8</t>
         </is>
       </c>
       <c r="H44" s="0" t="inlineStr">
         <is>
-          <t>3072.65</t>
-        </is>
-      </c>
-      <c r="J44" s="0" t="n">
-        <v>13.2787</v>
+          <t>5954.54</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -3036,17 +2902,17 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>24707.29</t>
+          <t>28826.25</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
-          <t>30859.7</t>
+          <t>29778.1</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>6152.41</t>
+          <t>951.849999999999</t>
         </is>
       </c>
       <c r="E45" s="0" t="inlineStr">
@@ -3056,21 +2922,18 @@
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>28552.78</t>
+          <t>24187.85</t>
         </is>
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>30901.7</t>
+          <t>29654.1</t>
         </is>
       </c>
       <c r="H45" s="0" t="inlineStr">
         <is>
-          <t>2348.92</t>
-        </is>
-      </c>
-      <c r="J45" s="0" t="n">
-        <v>13.2787</v>
+          <t>5466.25</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -3081,17 +2944,17 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>25157.94</t>
+          <t>29066.46</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
-          <t>31349.1</t>
+          <t>30009.7</t>
         </is>
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>6191.16</t>
+          <t>943.240000000002</t>
         </is>
       </c>
       <c r="E46" s="0" t="inlineStr">
@@ -3101,21 +2964,18 @@
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>29034.7</t>
+          <t>24643.86</t>
         </is>
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>31026.8</t>
+          <t>29577.2</t>
         </is>
       </c>
       <c r="H46" s="0" t="inlineStr">
         <is>
-          <t>1992.1</t>
-        </is>
-      </c>
-      <c r="J46" s="0" t="n">
-        <v>13.2787</v>
+          <t>4933.34</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -3126,17 +2986,17 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>25502.39</t>
+          <t>29230.01</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
         <is>
-          <t>31011.8</t>
+          <t>30033.5</t>
         </is>
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>5509.41</t>
+          <t>803.490000000002</t>
         </is>
       </c>
       <c r="E47" s="0" t="inlineStr">
@@ -3146,21 +3006,18 @@
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t>29402.23</t>
+          <t>25004.52</t>
         </is>
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>30896.8</t>
+          <t>29400</t>
         </is>
       </c>
       <c r="H47" s="0" t="inlineStr">
         <is>
-          <t>1494.57</t>
-        </is>
-      </c>
-      <c r="J47" s="0" t="n">
-        <v>13.2787</v>
+          <t>4395.48</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -3171,17 +3028,17 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>25758.62</t>
+          <t>29328.53</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
-          <t>30469.2</t>
+          <t>29635.3</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>4710.58</t>
+          <t>306.77</t>
         </is>
       </c>
       <c r="E48" s="0" t="inlineStr">
@@ -3191,21 +3048,18 @@
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>29669</t>
+          <t>25285.6</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>30545.7</t>
+          <t>29032.5</t>
         </is>
       </c>
       <c r="H48" s="0" t="inlineStr">
         <is>
-          <t>876.700000000001</t>
-        </is>
-      </c>
-      <c r="J48" s="0" t="n">
-        <v>13.2787</v>
+          <t>3746.9</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -3216,17 +3070,17 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>25905.64</t>
+          <t>29330.27</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
         <is>
-          <t>29753.8</t>
+          <t>29013.7</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>3848.16</t>
+          <t>-316.57</t>
         </is>
       </c>
       <c r="E49" s="0" t="inlineStr">
@@ -3236,21 +3090,18 @@
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>29817.8</t>
+          <t>25461.08</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>29860.2</t>
+          <t>28610.6</t>
         </is>
       </c>
       <c r="H49" s="0" t="inlineStr">
         <is>
-          <t>42.4000000000015</t>
-        </is>
-      </c>
-      <c r="J49" s="0" t="n">
-        <v>13.2787</v>
+          <t>3149.52</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -3261,17 +3112,17 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>25998.98</t>
+          <t>29273.75</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
         <is>
-          <t>29347.3</t>
+          <t>28670.1</t>
         </is>
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>3348.32</t>
+          <t>-603.650000000001</t>
         </is>
       </c>
       <c r="E50" s="0" t="inlineStr">
@@ -3281,21 +3132,18 @@
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>29885.5</t>
+          <t>25559.19</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>29321.3</t>
+          <t>28030.6</t>
         </is>
       </c>
       <c r="H50" s="0" t="inlineStr">
         <is>
-          <t>-564.200000000001</t>
-        </is>
-      </c>
-      <c r="J50" s="0" t="n">
-        <v>13.2787</v>
+          <t>2471.41</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -3306,17 +3154,17 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>26011.81</t>
+          <t>29170.3</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
         <is>
-          <t>29079.8</t>
+          <t>28712.3</t>
         </is>
       </c>
       <c r="D51" s="0" t="inlineStr">
         <is>
-          <t>3067.99</t>
+          <t>-458</t>
         </is>
       </c>
       <c r="E51" s="0" t="inlineStr">
@@ -3326,21 +3174,18 @@
       </c>
       <c r="F51" s="0" t="inlineStr">
         <is>
-          <t>29856.63</t>
+          <t>25574.55</t>
         </is>
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>29027.6</t>
+          <t>27920.3</t>
         </is>
       </c>
       <c r="H51" s="0" t="inlineStr">
         <is>
-          <t>-829.030000000002</t>
-        </is>
-      </c>
-      <c r="J51" s="0" t="n">
-        <v>13.2787</v>
+          <t>2345.75</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -3351,17 +3196,17 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>25930.48</t>
+          <t>29061.22</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
         <is>
-          <t>28852.8</t>
+          <t>29129.9</t>
         </is>
       </c>
       <c r="D52" s="0" t="inlineStr">
         <is>
-          <t>2922.32</t>
+          <t>68.6800000000003</t>
         </is>
       </c>
       <c r="E52" s="0" t="inlineStr">
@@ -3371,21 +3216,18 @@
       </c>
       <c r="F52" s="0" t="inlineStr">
         <is>
-          <t>29702.8</t>
+          <t>25537.16</t>
         </is>
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>28739.9</t>
+          <t>27731.5</t>
         </is>
       </c>
       <c r="H52" s="0" t="inlineStr">
         <is>
-          <t>-962.899999999998</t>
-        </is>
-      </c>
-      <c r="J52" s="0" t="n">
-        <v>13.2787</v>
+          <t>2194.34</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -3396,17 +3238,17 @@
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>25758.47</t>
+          <t>28865.18</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
         <is>
-          <t>28658.4</t>
+          <t>29348.9</t>
         </is>
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>2899.93</t>
+          <t>483.720000000001</t>
         </is>
       </c>
       <c r="E53" s="0" t="inlineStr">
@@ -3416,21 +3258,18 @@
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>29457.29</t>
+          <t>25429.22</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>28561.7</t>
+          <t>27760.2</t>
         </is>
       </c>
       <c r="H53" s="0" t="inlineStr">
         <is>
-          <t>-895.59</t>
-        </is>
-      </c>
-      <c r="J53" s="0" t="n">
-        <v>13.2787</v>
+          <t>2330.98</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -3441,17 +3280,17 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>25513.77</t>
+          <t>28663.39</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
         <is>
-          <t>28602.2</t>
+          <t>29564.9</t>
         </is>
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>3088.43</t>
+          <t>901.510000000002</t>
         </is>
       </c>
       <c r="E54" s="0" t="inlineStr">
@@ -3461,21 +3300,18 @@
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>29120.26</t>
+          <t>25286.9</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>28532.2</t>
+          <t>27785.8</t>
         </is>
       </c>
       <c r="H54" s="0" t="inlineStr">
         <is>
-          <t>-588.059999999998</t>
-        </is>
-      </c>
-      <c r="J54" s="0" t="n">
-        <v>13.2787</v>
+          <t>2498.9</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -3486,17 +3322,17 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>25177.46</t>
+          <t>28408.38</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
         <is>
-          <t>28622.2</t>
+          <t>29591.9</t>
         </is>
       </c>
       <c r="D55" s="0" t="inlineStr">
         <is>
-          <t>3444.74</t>
+          <t>1183.52</t>
         </is>
       </c>
       <c r="E55" s="0" t="inlineStr">
@@ -3506,21 +3342,18 @@
       </c>
       <c r="F55" s="0" t="inlineStr">
         <is>
-          <t>28677.98</t>
+          <t>25075.69</t>
         </is>
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>28403.5</t>
+          <t>27704.1</t>
         </is>
       </c>
       <c r="H55" s="0" t="inlineStr">
         <is>
-          <t>-274.48</t>
-        </is>
-      </c>
-      <c r="J55" s="0" t="n">
-        <v>13.2787</v>
+          <t>2628.41</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -3531,17 +3364,17 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>24756.84</t>
+          <t>28090.45</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
         <is>
-          <t>28887.1</t>
+          <t>29769.8</t>
         </is>
       </c>
       <c r="D56" s="0" t="inlineStr">
         <is>
-          <t>4130.26</t>
+          <t>1679.35</t>
         </is>
       </c>
       <c r="E56" s="0" t="inlineStr">
@@ -3551,21 +3384,18 @@
       </c>
       <c r="F56" s="0" t="inlineStr">
         <is>
-          <t>28141.35</t>
+          <t>24787.72</t>
         </is>
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>28426.5</t>
+          <t>27678.7</t>
         </is>
       </c>
       <c r="H56" s="0" t="inlineStr">
         <is>
-          <t>285.150000000001</t>
-        </is>
-      </c>
-      <c r="J56" s="0" t="n">
-        <v>13.2787</v>
+          <t>2890.98</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -3576,17 +3406,17 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>24260.24</t>
+          <t>27749.89</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
         <is>
-          <t>29184.5</t>
+          <t>29946.8</t>
         </is>
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>4924.26</t>
+          <t>2196.91</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
@@ -3596,21 +3426,18 @@
       </c>
       <c r="F57" s="0" t="inlineStr">
         <is>
-          <t>27511.11</t>
+          <t>24465.34</t>
         </is>
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>28819.2</t>
+          <t>27788.3</t>
         </is>
       </c>
       <c r="H57" s="0" t="inlineStr">
         <is>
-          <t>1308.09</t>
-        </is>
-      </c>
-      <c r="J57" s="0" t="n">
-        <v>13.2787</v>
+          <t>3322.96</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -3621,17 +3448,17 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>23643.19</t>
+          <t>27315.77</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
         <is>
-          <t>29654.7</t>
+          <t>30204.2</t>
         </is>
       </c>
       <c r="D58" s="0" t="inlineStr">
         <is>
-          <t>6011.51</t>
+          <t>2888.43</t>
         </is>
       </c>
       <c r="E58" s="0" t="inlineStr">
@@ -3641,21 +3468,18 @@
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>26783.53</t>
+          <t>24047.08</t>
         </is>
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>29100.4</t>
+          <t>27931</t>
         </is>
       </c>
       <c r="H58" s="0" t="inlineStr">
         <is>
-          <t>2316.87</t>
-        </is>
-      </c>
-      <c r="J58" s="0" t="n">
-        <v>13.2787</v>
+          <t>3883.92</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -3666,17 +3490,17 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>22934.6</t>
+          <t>26776.99</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
         <is>
-          <t>30015.8</t>
+          <t>30377.7</t>
         </is>
       </c>
       <c r="D59" s="0" t="inlineStr">
         <is>
-          <t>7081.2</t>
+          <t>3600.71</t>
         </is>
       </c>
       <c r="E59" s="0" t="inlineStr">
@@ -3686,21 +3510,18 @@
       </c>
       <c r="F59" s="0" t="inlineStr">
         <is>
-          <t>25970.33</t>
+          <t>23535.41</t>
         </is>
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>29378.8</t>
+          <t>28252.9</t>
         </is>
       </c>
       <c r="H59" s="0" t="inlineStr">
         <is>
-          <t>3408.47</t>
-        </is>
-      </c>
-      <c r="J59" s="0" t="n">
-        <v>13.2787</v>
+          <t>4717.49</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -3711,17 +3532,17 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>22130.85</t>
+          <t>26121.56</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
         <is>
-          <t>30206.1</t>
+          <t>30601</t>
         </is>
       </c>
       <c r="D60" s="0" t="inlineStr">
         <is>
-          <t>8075.25</t>
+          <t>4479.44</t>
         </is>
       </c>
       <c r="E60" s="0" t="inlineStr">
@@ -3731,21 +3552,18 @@
       </c>
       <c r="F60" s="0" t="inlineStr">
         <is>
-          <t>25069.1</t>
+          <t>22947.15</t>
         </is>
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>30030.8</t>
+          <t>28526</t>
         </is>
       </c>
       <c r="H60" s="0" t="inlineStr">
         <is>
-          <t>4961.7</t>
-        </is>
-      </c>
-      <c r="J60" s="0" t="n">
-        <v>13.2787</v>
+          <t>5578.85</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -3756,17 +3574,17 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>21267.57</t>
+          <t>25420.97</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
         <is>
-          <t>30429</t>
+          <t>30849</t>
         </is>
       </c>
       <c r="D61" s="0" t="inlineStr">
         <is>
-          <t>9161.43</t>
+          <t>5428.03</t>
         </is>
       </c>
       <c r="E61" s="0" t="inlineStr">
@@ -3776,21 +3594,18 @@
       </c>
       <c r="F61" s="0" t="inlineStr">
         <is>
-          <t>24136.94</t>
+          <t>22310.33</t>
         </is>
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>30272</t>
+          <t>28907.6</t>
         </is>
       </c>
       <c r="H61" s="0" t="inlineStr">
         <is>
-          <t>6135.06</t>
-        </is>
-      </c>
-      <c r="J61" s="0" t="n">
-        <v>13.2787</v>
+          <t>6597.27</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -3801,17 +3616,17 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>20272.59</t>
+          <t>24571.61</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
         <is>
-          <t>30758.5</t>
+          <t>31263.8</t>
         </is>
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>10485.91</t>
+          <t>6692.19</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
@@ -3821,21 +3636,18 @@
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>23109.04</t>
+          <t>21536.76</t>
         </is>
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>30627.7</t>
+          <t>29336.4</t>
         </is>
       </c>
       <c r="H62" s="0" t="inlineStr">
         <is>
-          <t>7518.66</t>
-        </is>
-      </c>
-      <c r="J62" s="0" t="n">
-        <v>18.8163</v>
+          <t>7799.64</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -3846,17 +3658,17 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>19200.89</t>
+          <t>23641.65</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
         <is>
-          <t>31034.6</t>
+          <t>31498.3</t>
         </is>
       </c>
       <c r="D63" s="0" t="inlineStr">
         <is>
-          <t>11833.71</t>
+          <t>7856.65</t>
         </is>
       </c>
       <c r="E63" s="0" t="inlineStr">
@@ -3866,21 +3678,18 @@
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>22017.27</t>
+          <t>20682.74</t>
         </is>
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>31155.6</t>
+          <t>29630</t>
         </is>
       </c>
       <c r="H63" s="0" t="inlineStr">
         <is>
-          <t>9138.33</t>
-        </is>
-      </c>
-      <c r="J63" s="0" t="n">
-        <v>47.0154</v>
+          <t>8947.26</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -3891,17 +3700,17 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>18063</t>
+          <t>22593.76</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
         <is>
-          <t>31381.8</t>
+          <t>31711</t>
         </is>
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>13318.8</t>
+          <t>9117.24</t>
         </is>
       </c>
       <c r="E64" s="0" t="inlineStr">
@@ -3911,21 +3720,18 @@
       </c>
       <c r="F64" s="0" t="inlineStr">
         <is>
-          <t>20872.96</t>
+          <t>19763.98</t>
         </is>
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>31388.2</t>
+          <t>29899.4</t>
         </is>
       </c>
       <c r="H64" s="0" t="inlineStr">
         <is>
-          <t>10515.24</t>
-        </is>
-      </c>
-      <c r="J64" s="0" t="n">
-        <v>45.0137</v>
+          <t>10135.42</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -3936,41 +3742,38 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>16901.38</t>
+          <t>21519.43</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
         <is>
-          <t>32037.9</t>
+          <t>31896.8</t>
         </is>
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>15136.52</t>
+          <t>10377.37</t>
         </is>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>19743.81</t>
+          <t>18828.16</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>31852.1</t>
+          <t>30248.2</t>
         </is>
       </c>
       <c r="H65" s="0" t="inlineStr">
         <is>
-          <t>12108.29</t>
-        </is>
-      </c>
-      <c r="J65" s="0" t="n">
-        <v>53.1473</v>
+          <t>11420.04</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -3981,41 +3784,38 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>15634.52</t>
+          <t>20311.39</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
         <is>
-          <t>32684.1</t>
+          <t>32167</t>
         </is>
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>17049.58</t>
+          <t>11855.61</t>
         </is>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>21.2</t>
         </is>
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>18513.28</t>
+          <t>17757.63</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>32259.6</t>
+          <t>30663.3</t>
         </is>
       </c>
       <c r="H66" s="0" t="inlineStr">
         <is>
-          <t>13746.32</t>
-        </is>
-      </c>
-      <c r="J66" s="0" t="n">
-        <v>185.8343</v>
+          <t>12905.67</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -4026,41 +3826,38 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>14318.96</t>
+          <t>19015.45</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
         <is>
-          <t>33412.4</t>
+          <t>32709.8</t>
         </is>
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>19093.44</t>
+          <t>13694.35</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>269</t>
         </is>
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>17250.02</t>
+          <t>16610.47</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>32779</t>
+          <t>31409.8</t>
         </is>
       </c>
       <c r="H67" s="0" t="inlineStr">
         <is>
-          <t>15528.98</t>
-        </is>
-      </c>
-      <c r="J67" s="0" t="n">
-        <v>205.2069</v>
+          <t>14799.33</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -4071,41 +3868,38 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>12961.45</t>
+          <t>17659.03</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
         <is>
-          <t>34079.6</t>
+          <t>33173.1</t>
         </is>
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>21118.15</t>
+          <t>15514.07</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>250</t>
         </is>
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>15968.58</t>
+          <t>15401.67</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>33838.3</t>
+          <t>32070</t>
         </is>
       </c>
       <c r="H68" s="0" t="inlineStr">
         <is>
-          <t>17869.72</t>
-        </is>
-      </c>
-      <c r="J68" s="0" t="n">
-        <v>251.2184</v>
+          <t>16668.33</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -4116,17 +3910,17 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>11619.58</t>
+          <t>16317.01</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
         <is>
-          <t>34881.9</t>
+          <t>33689.1</t>
         </is>
       </c>
       <c r="D69" s="0" t="inlineStr">
         <is>
-          <t>23262.32</t>
+          <t>17372.09</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
@@ -4136,21 +3930,18 @@
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>14694.6</t>
+          <t>14193.64</t>
         </is>
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>34820.2</t>
+          <t>32814.5</t>
         </is>
       </c>
       <c r="H69" s="0" t="inlineStr">
         <is>
-          <t>20125.6</t>
-        </is>
-      </c>
-      <c r="J69" s="0" t="n">
-        <v>274.669</v>
+          <t>18620.86</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -4161,41 +3952,38 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>10262.72</t>
+          <t>14893.59</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
         <is>
-          <t>35430.6</t>
+          <t>34105.8</t>
         </is>
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>25167.88</t>
+          <t>19212.21</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
-          <t>290</t>
+          <t>282</t>
         </is>
       </c>
       <c r="F70" s="0" t="inlineStr">
         <is>
-          <t>13415.04</t>
+          <t>12884.94</t>
         </is>
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>35572.4</t>
+          <t>33559</t>
         </is>
       </c>
       <c r="H70" s="0" t="inlineStr">
         <is>
-          <t>22157.36</t>
-        </is>
-      </c>
-      <c r="J70" s="0" t="n">
-        <v>285.7439</v>
+          <t>20674.06</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -4206,41 +3994,38 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>8918.38</t>
+          <t>13437.73</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
         <is>
-          <t>36287.4</t>
+          <t>34547.9</t>
         </is>
       </c>
       <c r="D71" s="0" t="inlineStr">
         <is>
-          <t>27369.02</t>
+          <t>21110.17</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>292</t>
         </is>
       </c>
       <c r="F71" s="0" t="inlineStr">
         <is>
-          <t>12169.86</t>
+          <t>11537.73</t>
         </is>
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>36383.2</t>
+          <t>34091.9</t>
         </is>
       </c>
       <c r="H71" s="0" t="inlineStr">
         <is>
-          <t>24213.34</t>
-        </is>
-      </c>
-      <c r="J71" s="0" t="n">
-        <v>298.2849</v>
+          <t>22554.17</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -4251,41 +4036,38 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>7663.38</t>
+          <t>12003.73</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
         <is>
-          <t>36903.4</t>
+          <t>34942.4</t>
         </is>
       </c>
       <c r="D72" s="0" t="inlineStr">
         <is>
-          <t>29240.02</t>
+          <t>22938.67</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>316</t>
         </is>
       </c>
       <c r="F72" s="0" t="inlineStr">
         <is>
-          <t>11018.28</t>
+          <t>10227.68</t>
         </is>
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>37157.8</t>
+          <t>34960.9</t>
         </is>
       </c>
       <c r="H72" s="0" t="inlineStr">
         <is>
-          <t>26139.52</t>
-        </is>
-      </c>
-      <c r="J72" s="0" t="n">
-        <v>317.1279</v>
+          <t>24733.22</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -4296,41 +4078,38 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>6572.52</t>
+          <t>10672.12</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
         <is>
-          <t>37312</t>
+          <t>35310.1</t>
         </is>
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>30739.48</t>
+          <t>24637.98</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
         <is>
-          <t>396</t>
+          <t>320</t>
         </is>
       </c>
       <c r="F73" s="0" t="inlineStr">
         <is>
-          <t>9993.63</t>
+          <t>9007.7</t>
         </is>
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>37858</t>
+          <t>35195.2</t>
         </is>
       </c>
       <c r="H73" s="0" t="inlineStr">
         <is>
-          <t>27864.37</t>
-        </is>
-      </c>
-      <c r="J73" s="0" t="n">
-        <v>318.9801</v>
+          <t>26187.5</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -4341,41 +4120,38 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>5650.38</t>
+          <t>9387.56</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
         <is>
-          <t>37720.6</t>
+          <t>35679.8</t>
         </is>
       </c>
       <c r="D74" s="0" t="inlineStr">
         <is>
-          <t>32070.22</t>
+          <t>26292.24</t>
         </is>
       </c>
       <c r="E74" s="0" t="inlineStr">
         <is>
-          <t>453</t>
+          <t>320</t>
         </is>
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>9097.89</t>
+          <t>7865.23</t>
         </is>
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>38483.9</t>
+          <t>35578.6</t>
         </is>
       </c>
       <c r="H74" s="0" t="inlineStr">
         <is>
-          <t>29386.01</t>
-        </is>
-      </c>
-      <c r="J74" s="0" t="n">
-        <v>325.152</v>
+          <t>27713.37</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -4386,41 +4162,38 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>4912.88</t>
+          <t>8189.77</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
         <is>
-          <t>38169.8</t>
+          <t>36190.3</t>
         </is>
       </c>
       <c r="D75" s="0" t="inlineStr">
         <is>
-          <t>33256.92</t>
+          <t>28000.53</t>
         </is>
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>330</t>
         </is>
       </c>
       <c r="F75" s="0" t="inlineStr">
         <is>
-          <t>8389.78</t>
+          <t>6796.37</t>
         </is>
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>39067.9</t>
+          <t>36127.6</t>
         </is>
       </c>
       <c r="H75" s="0" t="inlineStr">
         <is>
-          <t>30678.12</t>
-        </is>
-      </c>
-      <c r="J75" s="0" t="n">
-        <v>329.2145</v>
+          <t>29331.23</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -4431,41 +4204,38 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>4276.37</t>
+          <t>7136.51</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
         <is>
-          <t>38860.9</t>
+          <t>36675</t>
         </is>
       </c>
       <c r="D76" s="0" t="inlineStr">
         <is>
-          <t>34584.53</t>
+          <t>29538.49</t>
         </is>
       </c>
       <c r="E76" s="0" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>350</t>
         </is>
       </c>
       <c r="F76" s="0" t="inlineStr">
         <is>
-          <t>7762.36</t>
+          <t>5876.05</t>
         </is>
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>40007.8</t>
+          <t>36765.6</t>
         </is>
       </c>
       <c r="H76" s="0" t="inlineStr">
         <is>
-          <t>32245.44</t>
-        </is>
-      </c>
-      <c r="J76" s="0" t="n">
-        <v>329.2145</v>
+          <t>30889.55</t>
+        </is>
       </c>
     </row>
     <row r="77">
@@ -4476,41 +4246,38 @@
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>3947.43</t>
+          <t>6151.98</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
         <is>
-          <t>39344.6</t>
+          <t>37134.8</t>
         </is>
       </c>
       <c r="D77" s="0" t="inlineStr">
         <is>
-          <t>35397.17</t>
+          <t>30982.82</t>
         </is>
       </c>
       <c r="E77" s="0" t="inlineStr">
         <is>
-          <t>575</t>
+          <t>390</t>
         </is>
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>7389.39</t>
+          <t>5040.47</t>
         </is>
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>40528.2</t>
+          <t>37154.6</t>
         </is>
       </c>
       <c r="H77" s="0" t="inlineStr">
         <is>
-          <t>33138.81</t>
-        </is>
-      </c>
-      <c r="J77" s="0" t="n">
-        <v>344.9773</v>
+          <t>32114.13</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -4521,41 +4288,38 @@
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>3885.8</t>
+          <t>5491.58</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
         <is>
-          <t>39863.9</t>
+          <t>37497.4</t>
         </is>
       </c>
       <c r="D78" s="0" t="inlineStr">
         <is>
-          <t>35978.1</t>
+          <t>32005.82</t>
         </is>
       </c>
       <c r="E78" s="0" t="inlineStr">
         <is>
-          <t>914</t>
+          <t>398.4</t>
         </is>
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>7305.79</t>
+          <t>4537.12</t>
         </is>
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>41124</t>
+          <t>37545.6</t>
         </is>
       </c>
       <c r="H78" s="0" t="inlineStr">
         <is>
-          <t>33818.21</t>
-        </is>
-      </c>
-      <c r="J78" s="0" t="n">
-        <v>375.7242</v>
+          <t>33008.48</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -4566,41 +4330,38 @@
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>3929.42</t>
+          <t>5040.42</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
         <is>
-          <t>40140.4</t>
+          <t>37738.4</t>
         </is>
       </c>
       <c r="D79" s="0" t="inlineStr">
         <is>
-          <t>36210.98</t>
+          <t>32697.98</t>
         </is>
       </c>
       <c r="E79" s="0" t="inlineStr">
         <is>
-          <t>575</t>
+          <t>400</t>
         </is>
       </c>
       <c r="F79" s="0" t="inlineStr">
         <is>
-          <t>7336.31</t>
+          <t>4280.87</t>
         </is>
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>41399.8</t>
+          <t>37717.6</t>
         </is>
       </c>
       <c r="H79" s="0" t="inlineStr">
         <is>
-          <t>34063.49</t>
-        </is>
-      </c>
-      <c r="J79" s="0" t="n">
-        <v>375.7242</v>
+          <t>33436.73</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -4611,41 +4372,38 @@
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>4178.19</t>
+          <t>4760.39</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
         <is>
-          <t>40935.1</t>
+          <t>37979.5</t>
         </is>
       </c>
       <c r="D80" s="0" t="inlineStr">
         <is>
-          <t>36756.91</t>
+          <t>33219.11</t>
         </is>
       </c>
       <c r="E80" s="0" t="inlineStr">
         <is>
-          <t>1014</t>
+          <t>412</t>
         </is>
       </c>
       <c r="F80" s="0" t="inlineStr">
         <is>
-          <t>7536.42</t>
+          <t>4199.77</t>
         </is>
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>41602.7</t>
+          <t>37890.6</t>
         </is>
       </c>
       <c r="H80" s="0" t="inlineStr">
         <is>
-          <t>34066.28</t>
-        </is>
-      </c>
-      <c r="J80" s="0" t="n">
-        <v>346.73</v>
+          <t>33690.83</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -4656,41 +4414,38 @@
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>4531.82</t>
+          <t>4680.78</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
         <is>
-          <t>40520.4</t>
+          <t>38096.4</t>
         </is>
       </c>
       <c r="D81" s="0" t="inlineStr">
         <is>
-          <t>35988.58</t>
+          <t>33415.62</t>
         </is>
       </c>
       <c r="E81" s="0" t="inlineStr">
         <is>
-          <t>917</t>
+          <t>419</t>
         </is>
       </c>
       <c r="F81" s="0" t="inlineStr">
         <is>
-          <t>7906.8</t>
+          <t>4383.73</t>
         </is>
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>41724.5</t>
+          <t>38175.6</t>
         </is>
       </c>
       <c r="H81" s="0" t="inlineStr">
         <is>
-          <t>33817.7</t>
-        </is>
-      </c>
-      <c r="J81" s="0" t="n">
-        <v>331.1733</v>
+          <t>33791.87</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -4701,41 +4456,38 @@
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>4742.26</t>
+          <t>4546.31</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
         <is>
-          <t>40209.5</t>
+          <t>38238.2</t>
         </is>
       </c>
       <c r="D82" s="0" t="inlineStr">
         <is>
-          <t>35467.24</t>
+          <t>33691.89</t>
         </is>
       </c>
       <c r="E82" s="0" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>450</t>
         </is>
       </c>
       <c r="F82" s="0" t="inlineStr">
         <is>
-          <t>8093.36</t>
+          <t>4463.06</t>
         </is>
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>41602.7</t>
+          <t>38325.6</t>
         </is>
       </c>
       <c r="H82" s="0" t="inlineStr">
         <is>
-          <t>33509.34</t>
-        </is>
-      </c>
-      <c r="J82" s="0" t="n">
-        <v>331.1733</v>
+          <t>33862.54</t>
+        </is>
       </c>
     </row>
     <row r="83">
@@ -4746,41 +4498,38 @@
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>4929.86</t>
+          <t>4414.53</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
         <is>
-          <t>39747.9</t>
+          <t>38137.4</t>
         </is>
       </c>
       <c r="D83" s="0" t="inlineStr">
         <is>
-          <t>34818.04</t>
+          <t>33722.87</t>
         </is>
       </c>
       <c r="E83" s="0" t="inlineStr">
         <is>
-          <t>567</t>
+          <t>430</t>
         </is>
       </c>
       <c r="F83" s="0" t="inlineStr">
         <is>
-          <t>8290.77</t>
+          <t>4543.35</t>
         </is>
       </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
-          <t>41243.3</t>
+          <t>38034.6</t>
         </is>
       </c>
       <c r="H83" s="0" t="inlineStr">
         <is>
-          <t>32952.53</t>
-        </is>
-      </c>
-      <c r="J83" s="0" t="n">
-        <v>331.1733</v>
+          <t>33491.25</t>
+        </is>
       </c>
     </row>
     <row r="84">
@@ -4791,41 +4540,38 @@
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t>5122.95</t>
+          <t>4289.04</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
         <is>
-          <t>39528.3</t>
+          <t>37838.2</t>
         </is>
       </c>
       <c r="D84" s="0" t="inlineStr">
         <is>
-          <t>34405.35</t>
+          <t>33549.16</t>
         </is>
       </c>
       <c r="E84" s="0" t="inlineStr">
         <is>
-          <t>564</t>
+          <t>439</t>
         </is>
       </c>
       <c r="F84" s="0" t="inlineStr">
         <is>
-          <t>8465.92</t>
+          <t>4636.6</t>
         </is>
       </c>
       <c r="G84" s="0" t="inlineStr">
         <is>
-          <t>40743.3</t>
+          <t>37698.6</t>
         </is>
       </c>
       <c r="H84" s="0" t="inlineStr">
         <is>
-          <t>32277.38</t>
-        </is>
-      </c>
-      <c r="J84" s="0" t="n">
-        <v>329.2145</v>
+          <t>33062</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -4836,41 +4582,38 @@
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t>5320.15</t>
+          <t>4184.73</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
         <is>
-          <t>39550.5</t>
+          <t>37264.8</t>
         </is>
       </c>
       <c r="D85" s="0" t="inlineStr">
         <is>
-          <t>34230.35</t>
+          <t>33080.07</t>
         </is>
       </c>
       <c r="E85" s="0" t="inlineStr">
         <is>
-          <t>459</t>
+          <t>420</t>
         </is>
       </c>
       <c r="F85" s="0" t="inlineStr">
         <is>
-          <t>8669.2</t>
+          <t>4765.39</t>
         </is>
       </c>
       <c r="G85" s="0" t="inlineStr">
         <is>
-          <t>40441.4</t>
+          <t>37293.6</t>
         </is>
       </c>
       <c r="H85" s="0" t="inlineStr">
         <is>
-          <t>31772.2</t>
-        </is>
-      </c>
-      <c r="J85" s="0" t="n">
-        <v>329.2145</v>
+          <t>32528.21</t>
+        </is>
       </c>
     </row>
     <row r="86">
@@ -4881,41 +4624,38 @@
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t>5466.43</t>
+          <t>4031.97</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
         <is>
-          <t>39326.8</t>
+          <t>36788.8</t>
         </is>
       </c>
       <c r="D86" s="0" t="inlineStr">
         <is>
-          <t>33860.37</t>
+          <t>32756.83</t>
         </is>
       </c>
       <c r="E86" s="0" t="inlineStr">
         <is>
-          <t>920</t>
+          <t>450</t>
         </is>
       </c>
       <c r="F86" s="0" t="inlineStr">
         <is>
-          <t>8806.56</t>
+          <t>4857.26</t>
         </is>
       </c>
       <c r="G86" s="0" t="inlineStr">
         <is>
-          <t>40024.1</t>
+          <t>36931.6</t>
         </is>
       </c>
       <c r="H86" s="0" t="inlineStr">
         <is>
-          <t>31217.54</t>
-        </is>
-      </c>
-      <c r="J86" s="0" t="n">
-        <v>329.2145</v>
+          <t>32074.34</t>
+        </is>
       </c>
     </row>
     <row r="87">
@@ -4926,41 +4666,38 @@
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>5628.55</t>
+          <t>3895.28</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
         <is>
-          <t>38560</t>
+          <t>36216.6</t>
         </is>
       </c>
       <c r="D87" s="0" t="inlineStr">
         <is>
-          <t>32931.45</t>
+          <t>32321.32</t>
         </is>
       </c>
       <c r="E87" s="0" t="inlineStr">
         <is>
-          <t>914</t>
+          <t>448</t>
         </is>
       </c>
       <c r="F87" s="0" t="inlineStr">
         <is>
-          <t>8966.55</t>
+          <t>4963.55</t>
         </is>
       </c>
       <c r="G87" s="0" t="inlineStr">
         <is>
-          <t>39438.4</t>
+          <t>36425.6</t>
         </is>
       </c>
       <c r="H87" s="0" t="inlineStr">
         <is>
-          <t>30471.85</t>
-        </is>
-      </c>
-      <c r="J87" s="0" t="n">
-        <v>328.1401</v>
+          <t>31462.05</t>
+        </is>
       </c>
     </row>
     <row r="88">
@@ -4971,41 +4708,38 @@
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t>5796.83</t>
+          <t>3759.68</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
         <is>
-          <t>37967.9</t>
+          <t>35623.5</t>
         </is>
       </c>
       <c r="D88" s="0" t="inlineStr">
         <is>
-          <t>32171.07</t>
+          <t>31863.82</t>
         </is>
       </c>
       <c r="E88" s="0" t="inlineStr">
         <is>
-          <t>567</t>
+          <t>410</t>
         </is>
       </c>
       <c r="F88" s="0" t="inlineStr">
         <is>
-          <t>9138.35</t>
+          <t>5084.41</t>
         </is>
       </c>
       <c r="G88" s="0" t="inlineStr">
         <is>
-          <t>38929</t>
+          <t>35901.6</t>
         </is>
       </c>
       <c r="H88" s="0" t="inlineStr">
         <is>
-          <t>29790.65</t>
-        </is>
-      </c>
-      <c r="J88" s="0" t="n">
-        <v>325.152</v>
+          <t>30817.19</t>
+        </is>
       </c>
     </row>
     <row r="89">
@@ -5016,41 +4750,38 @@
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t>5974.14</t>
+          <t>3642.94</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
         <is>
-          <t>37410.4</t>
+          <t>35079.1</t>
         </is>
       </c>
       <c r="D89" s="0" t="inlineStr">
         <is>
-          <t>31436.26</t>
+          <t>31436.16</t>
         </is>
       </c>
       <c r="E89" s="0" t="inlineStr">
         <is>
-          <t>460.01</t>
+          <t>400</t>
         </is>
       </c>
       <c r="F89" s="0" t="inlineStr">
         <is>
-          <t>9324.12</t>
+          <t>5217.89</t>
         </is>
       </c>
       <c r="G89" s="0" t="inlineStr">
         <is>
-          <t>38308.1</t>
+          <t>35353.6</t>
         </is>
       </c>
       <c r="H89" s="0" t="inlineStr">
         <is>
-          <t>28983.98</t>
-        </is>
-      </c>
-      <c r="J89" s="0" t="n">
-        <v>320.5447</v>
+          <t>30135.71</t>
+        </is>
       </c>
     </row>
     <row r="90">
@@ -5061,41 +4792,38 @@
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t>6147.07</t>
+          <t>3531.59</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
         <is>
-          <t>36925.9</t>
+          <t>34489.1</t>
         </is>
       </c>
       <c r="D90" s="0" t="inlineStr">
         <is>
-          <t>30778.83</t>
+          <t>30957.51</t>
         </is>
       </c>
       <c r="E90" s="0" t="inlineStr">
         <is>
-          <t>395</t>
+          <t>399</t>
         </is>
       </c>
       <c r="F90" s="0" t="inlineStr">
         <is>
-          <t>9496.83</t>
+          <t>5359.38</t>
         </is>
       </c>
       <c r="G90" s="0" t="inlineStr">
         <is>
-          <t>37654.1</t>
+          <t>34787.6</t>
         </is>
       </c>
       <c r="H90" s="0" t="inlineStr">
         <is>
-          <t>28157.27</t>
-        </is>
-      </c>
-      <c r="J90" s="0" t="n">
-        <v>316.4748</v>
+          <t>29428.22</t>
+        </is>
       </c>
     </row>
     <row r="91">
@@ -5106,41 +4834,38 @@
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t>6318.56</t>
+          <t>3423.2</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
         <is>
-          <t>36580.1</t>
+          <t>33978.6</t>
         </is>
       </c>
       <c r="D91" s="0" t="inlineStr">
         <is>
-          <t>30261.54</t>
+          <t>30555.4</t>
         </is>
       </c>
       <c r="E91" s="0" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>398.4</t>
         </is>
       </c>
       <c r="F91" s="0" t="inlineStr">
         <is>
-          <t>9661.8</t>
+          <t>5514.9</t>
         </is>
       </c>
       <c r="G91" s="0" t="inlineStr">
         <is>
-          <t>37289.9</t>
+          <t>34238.6</t>
         </is>
       </c>
       <c r="H91" s="0" t="inlineStr">
         <is>
-          <t>27628.1</t>
-        </is>
-      </c>
-      <c r="J91" s="0" t="n">
-        <v>316.4748</v>
+          <t>28723.7</t>
+        </is>
       </c>
     </row>
     <row r="92">
@@ -5151,41 +4876,38 @@
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t>6473.47</t>
+          <t>3317.79</t>
         </is>
       </c>
       <c r="C92" s="0" t="inlineStr">
         <is>
-          <t>36062.4</t>
+          <t>33545.6</t>
         </is>
       </c>
       <c r="D92" s="0" t="inlineStr">
         <is>
-          <t>29588.93</t>
+          <t>30227.81</t>
         </is>
       </c>
       <c r="E92" s="0" t="inlineStr">
         <is>
-          <t>335</t>
+          <t>395</t>
         </is>
       </c>
       <c r="F92" s="0" t="inlineStr">
         <is>
-          <t>9819.35</t>
+          <t>5667.96</t>
         </is>
       </c>
       <c r="G92" s="0" t="inlineStr">
         <is>
-          <t>36889.5</t>
+          <t>33692.6</t>
         </is>
       </c>
       <c r="H92" s="0" t="inlineStr">
         <is>
-          <t>27070.15</t>
-        </is>
-      </c>
-      <c r="J92" s="0" t="n">
-        <v>316.4748</v>
+          <t>28024.64</t>
+        </is>
       </c>
     </row>
     <row r="93">
@@ -5196,41 +4918,38 @@
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t>6634.12</t>
+          <t>3221.04</t>
         </is>
       </c>
       <c r="C93" s="0" t="inlineStr">
         <is>
-          <t>35682</t>
+          <t>33112.5</t>
         </is>
       </c>
       <c r="D93" s="0" t="inlineStr">
         <is>
-          <t>29047.88</t>
+          <t>29891.46</t>
         </is>
       </c>
       <c r="E93" s="0" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>390</t>
         </is>
       </c>
       <c r="F93" s="0" t="inlineStr">
         <is>
-          <t>9982</t>
+          <t>5835.17</t>
         </is>
       </c>
       <c r="G93" s="0" t="inlineStr">
         <is>
-          <t>36413.8</t>
+          <t>33123.6</t>
         </is>
       </c>
       <c r="H93" s="0" t="inlineStr">
         <is>
-          <t>26431.8</t>
-        </is>
-      </c>
-      <c r="J93" s="0" t="n">
-        <v>314.6226</v>
+          <t>27288.43</t>
+        </is>
       </c>
     </row>
     <row r="94">
@@ -5241,41 +4960,38 @@
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t>6755.51</t>
+          <t>3132.29</t>
         </is>
       </c>
       <c r="C94" s="0" t="inlineStr">
         <is>
-          <t>35303.6</t>
+          <t>32631.8</t>
         </is>
       </c>
       <c r="D94" s="0" t="inlineStr">
         <is>
-          <t>28548.09</t>
+          <t>29499.51</t>
         </is>
       </c>
       <c r="E94" s="0" t="inlineStr">
         <is>
-          <t>314</t>
+          <t>380</t>
         </is>
       </c>
       <c r="F94" s="0" t="inlineStr">
         <is>
-          <t>10122.38</t>
+          <t>6008.48</t>
         </is>
       </c>
       <c r="G94" s="0" t="inlineStr">
         <is>
-          <t>36014.5</t>
+          <t>32557.6</t>
         </is>
       </c>
       <c r="H94" s="0" t="inlineStr">
         <is>
-          <t>25892.12</t>
-        </is>
-      </c>
-      <c r="J94" s="0" t="n">
-        <v>313.588</v>
+          <t>26549.12</t>
+        </is>
       </c>
     </row>
     <row r="95">
@@ -5286,41 +5002,38 @@
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t>6873.73</t>
+          <t>3047.4</t>
         </is>
       </c>
       <c r="C95" s="0" t="inlineStr">
         <is>
-          <t>35297.2</t>
+          <t>32495</t>
         </is>
       </c>
       <c r="D95" s="0" t="inlineStr">
         <is>
-          <t>28423.47</t>
+          <t>29447.6</t>
         </is>
       </c>
       <c r="E95" s="0" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>360</t>
         </is>
       </c>
       <c r="F95" s="0" t="inlineStr">
         <is>
-          <t>10233.54</t>
+          <t>6190.54</t>
         </is>
       </c>
       <c r="G95" s="0" t="inlineStr">
         <is>
-          <t>35843.8</t>
+          <t>32423.6</t>
         </is>
       </c>
       <c r="H95" s="0" t="inlineStr">
         <is>
-          <t>25610.26</t>
-        </is>
-      </c>
-      <c r="J95" s="0" t="n">
-        <v>307.9694</v>
+          <t>26233.06</t>
+        </is>
       </c>
     </row>
     <row r="96">
@@ -5331,41 +5044,38 @@
       </c>
       <c r="B96" s="0" t="inlineStr">
         <is>
-          <t>6994.9</t>
+          <t>2966.36</t>
         </is>
       </c>
       <c r="C96" s="0" t="inlineStr">
         <is>
-          <t>34881.8</t>
+          <t>32313.5</t>
         </is>
       </c>
       <c r="D96" s="0" t="inlineStr">
         <is>
-          <t>27886.9</t>
+          <t>29347.14</t>
         </is>
       </c>
       <c r="E96" s="0" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>396</t>
         </is>
       </c>
       <c r="F96" s="0" t="inlineStr">
         <is>
-          <t>10348.63</t>
+          <t>6368.69</t>
         </is>
       </c>
       <c r="G96" s="0" t="inlineStr">
         <is>
-          <t>35569.7</t>
+          <t>32294.6</t>
         </is>
       </c>
       <c r="H96" s="0" t="inlineStr">
         <is>
-          <t>25221.07</t>
-        </is>
-      </c>
-      <c r="J96" s="0" t="n">
-        <v>307.9694</v>
+          <t>25925.91</t>
+        </is>
       </c>
     </row>
     <row r="97">
@@ -5376,41 +5086,38 @@
       </c>
       <c r="B97" s="0" t="inlineStr">
         <is>
-          <t>7059.09</t>
+          <t>2894.38</t>
         </is>
       </c>
       <c r="C97" s="0" t="inlineStr">
         <is>
-          <t>34849.5</t>
+          <t>32353.4</t>
         </is>
       </c>
       <c r="D97" s="0" t="inlineStr">
         <is>
-          <t>27790.41</t>
+          <t>29459.02</t>
         </is>
       </c>
       <c r="E97" s="0" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>396</t>
         </is>
       </c>
       <c r="F97" s="0" t="inlineStr">
         <is>
-          <t>10473.13</t>
+          <t>6566.93</t>
         </is>
       </c>
       <c r="G97" s="0" t="inlineStr">
         <is>
-          <t>35447.4</t>
+          <t>32412.6</t>
         </is>
       </c>
       <c r="H97" s="0" t="inlineStr">
         <is>
-          <t>24974.27</t>
-        </is>
-      </c>
-      <c r="J97" s="0" t="n">
-        <v>297.5983</v>
+          <t>25845.67</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>